<commit_message>
Centralize market state and migrate engines to shared context
</commit_message>
<xml_diff>
--- a/data/exports/dev-portfolio_intelligence.xlsx
+++ b/data/exports/dev-portfolio_intelligence.xlsx
@@ -1646,7 +1646,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2030</v>
+        <v>2010</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1662,7 +1662,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BZ=F</t>
+          <t>^VIX</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1960</v>
+        <v>1940</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1680,14 +1680,14 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>bullish trend, potentially oversold</t>
+          <t>bullish trend</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CL=F</t>
+          <t>BZ=F</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1950</v>
+        <v>1930</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1705,14 +1705,14 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>bullish trend</t>
+          <t>bullish trend, potentially oversold</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SI=F</t>
+          <t>CL=F</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1940</v>
+        <v>1910</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>^VIX</t>
+          <t>SI=F</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1930</v>
+        <v>1910</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1890</v>
+        <v>1880</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1840</v>
+        <v>1860</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -3155,7 +3155,7 @@
         <v>0.7716</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7389</v>
+        <v>0.7305</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -3185,26 +3185,26 @@
         <v>0.5</v>
       </c>
       <c r="R2" t="n">
-        <v>0.5</v>
+        <v>0.4436</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BZ=F</t>
+          <t>^VIX</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>93.55999755859375</v>
+        <v>16.95000076293945</v>
       </c>
       <c r="C3" t="n">
-        <v>104.7419999694824</v>
+        <v>20.32680011749268</v>
       </c>
       <c r="D3" t="n">
-        <v>76.57019987106324</v>
+        <v>18.37480008125305</v>
       </c>
       <c r="E3" t="n">
-        <v>39.85259342193125</v>
+        <v>48.98279176848897</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -3213,13 +3213,13 @@
         <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>0.8007</v>
+        <v>0.7551</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6015</v>
+        <v>0.5102</v>
       </c>
       <c r="J3" t="n">
-        <v>0.7134</v>
+        <v>0.7045</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -3249,26 +3249,26 @@
         <v>0.5</v>
       </c>
       <c r="R3" t="n">
-        <v>0.5</v>
+        <v>0.5318000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CL=F</t>
+          <t>BZ=F</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>90.16000366210938</v>
+        <v>93.55999755859375</v>
       </c>
       <c r="C4" t="n">
-        <v>98.21839981079101</v>
+        <v>104.7419999694824</v>
       </c>
       <c r="D4" t="n">
-        <v>71.80154985427856</v>
+        <v>76.57019987106324</v>
       </c>
       <c r="E4" t="n">
-        <v>43.05869679501007</v>
+        <v>39.85259342193125</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -3277,13 +3277,13 @@
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7847</v>
+        <v>0.8007</v>
       </c>
       <c r="I4" t="n">
-        <v>0.5694</v>
+        <v>0.6015</v>
       </c>
       <c r="J4" t="n">
-        <v>0.7086</v>
+        <v>0.7004</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -3313,26 +3313,26 @@
         <v>0.5</v>
       </c>
       <c r="R4" t="n">
-        <v>0.5</v>
+        <v>0.4135</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SI=F</t>
+          <t>CL=F</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>74.77999877929688</v>
+        <v>90.16000366210938</v>
       </c>
       <c r="C5" t="n">
-        <v>75.93557952880859</v>
+        <v>98.21839981079101</v>
       </c>
       <c r="D5" t="n">
-        <v>65.23656997680663</v>
+        <v>71.80154985427856</v>
       </c>
       <c r="E5" t="n">
-        <v>46.71263911332996</v>
+        <v>43.05869679501007</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -3341,13 +3341,13 @@
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>0.7664</v>
+        <v>0.7847</v>
       </c>
       <c r="I5" t="n">
-        <v>0.5329</v>
+        <v>0.5694</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7030999999999999</v>
+        <v>0.6949</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -3377,26 +3377,26 @@
         <v>0.5</v>
       </c>
       <c r="R5" t="n">
-        <v>0.5</v>
+        <v>0.4084</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>^VIX</t>
+          <t>SI=F</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16.95000076293945</v>
+        <v>74.77999877929688</v>
       </c>
       <c r="C6" t="n">
-        <v>20.32680011749268</v>
+        <v>75.93557952880859</v>
       </c>
       <c r="D6" t="n">
-        <v>18.37480008125305</v>
+        <v>65.23656997680663</v>
       </c>
       <c r="E6" t="n">
-        <v>48.98279176848897</v>
+        <v>46.71263911332996</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -3405,13 +3405,13 @@
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7551</v>
+        <v>0.7664</v>
       </c>
       <c r="I6" t="n">
-        <v>0.5102</v>
+        <v>0.5329</v>
       </c>
       <c r="J6" t="n">
-        <v>0.6997</v>
+        <v>0.694</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -3441,7 +3441,7 @@
         <v>0.5</v>
       </c>
       <c r="R6" t="n">
-        <v>0.5</v>
+        <v>0.4394</v>
       </c>
     </row>
     <row r="7">
@@ -3475,7 +3475,7 @@
         <v>0.4247</v>
       </c>
       <c r="J7" t="n">
-        <v>0.6869</v>
+        <v>0.6825</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -3505,7 +3505,7 @@
         <v>0.5</v>
       </c>
       <c r="R7" t="n">
-        <v>0.5</v>
+        <v>0.4709</v>
       </c>
     </row>
     <row r="8">
@@ -3539,7 +3539,7 @@
         <v>0.3202</v>
       </c>
       <c r="J8" t="n">
-        <v>0.6712</v>
+        <v>0.6758</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -3569,7 +3569,7 @@
         <v>0.5</v>
       </c>
       <c r="R8" t="n">
-        <v>0.5</v>
+        <v>0.5305</v>
       </c>
     </row>
     <row r="9">
@@ -3603,7 +3603,7 @@
         <v>0.309</v>
       </c>
       <c r="J9" t="n">
-        <v>0.3695</v>
+        <v>0.3676</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -3633,7 +3633,7 @@
         <v>0.5</v>
       </c>
       <c r="R9" t="n">
-        <v>0.5</v>
+        <v>0.4872</v>
       </c>
     </row>
   </sheetData>
@@ -3712,7 +3712,7 @@
         <v>4462.89990234375</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7389</v>
+        <v>0.7305</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -3737,7 +3737,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BZ=F</t>
+          <t>^VIX</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3746,10 +3746,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>93.55999755859375</v>
+        <v>16.95000076293945</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7134</v>
+        <v>0.7045</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -3760,21 +3760,21 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>39.85259342193125</v>
+        <v>48.98279176848897</v>
       </c>
       <c r="H3" t="n">
         <v>0.6546</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>bullish trend, potentially oversold</t>
+          <t>bullish trend</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CL=F</t>
+          <t>BZ=F</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3783,10 +3783,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>90.16000366210938</v>
+        <v>93.55999755859375</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7086</v>
+        <v>0.7004</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -3797,21 +3797,21 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>43.05869679501007</v>
+        <v>39.85259342193125</v>
       </c>
       <c r="H4" t="n">
         <v>0.6546</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>bullish trend</t>
+          <t>bullish trend, potentially oversold</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SI=F</t>
+          <t>CL=F</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3820,10 +3820,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>74.77999877929688</v>
+        <v>90.16000366210938</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7030999999999999</v>
+        <v>0.6949</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -3834,7 +3834,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>46.71263911332996</v>
+        <v>43.05869679501007</v>
       </c>
       <c r="H5" t="n">
         <v>0.6546</v>
@@ -3848,7 +3848,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>^VIX</t>
+          <t>SI=F</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3857,10 +3857,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16.95000076293945</v>
+        <v>74.77999877929688</v>
       </c>
       <c r="D6" t="n">
-        <v>0.6997</v>
+        <v>0.694</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -3871,7 +3871,7 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>48.98279176848897</v>
+        <v>46.71263911332996</v>
       </c>
       <c r="H6" t="n">
         <v>0.6546</v>
@@ -3897,7 +3897,7 @@
         <v>6.335000038146973</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6869</v>
+        <v>0.6825</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -3934,7 +3934,7 @@
         <v>99.22200012207031</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6712</v>
+        <v>0.6758</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -3971,7 +3971,7 @@
         <v>3.117000102996826</v>
       </c>
       <c r="D9" t="n">
-        <v>0.3695</v>
+        <v>0.3676</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -4081,7 +4081,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.7389</v>
+        <v>0.7305</v>
       </c>
       <c r="D2" t="n">
         <v>0.5</v>
@@ -4090,10 +4090,10 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>2.03</v>
+        <v>2.01</v>
       </c>
       <c r="G2" t="n">
-        <v>2030</v>
+        <v>2010</v>
       </c>
       <c r="H2" t="n">
         <v>4462.89990234375</v>
@@ -4118,7 +4118,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BZ=F</t>
+          <t>^VIX</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4127,7 +4127,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.7134</v>
+        <v>0.7045</v>
       </c>
       <c r="D3" t="n">
         <v>0.5</v>
@@ -4136,16 +4136,16 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1.96</v>
+        <v>1.94</v>
       </c>
       <c r="G3" t="n">
-        <v>1960</v>
+        <v>1940</v>
       </c>
       <c r="H3" t="n">
-        <v>93.55999755859375</v>
+        <v>16.95000076293945</v>
       </c>
       <c r="I3" t="n">
-        <v>20.95</v>
+        <v>114.45</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -4157,14 +4157,14 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>bullish trend, potentially oversold</t>
+          <t>bullish trend</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CL=F</t>
+          <t>BZ=F</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.7086</v>
+        <v>0.7004</v>
       </c>
       <c r="D4" t="n">
         <v>0.5</v>
@@ -4182,16 +4182,16 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>1.95</v>
+        <v>1.93</v>
       </c>
       <c r="G4" t="n">
-        <v>1950</v>
+        <v>1930</v>
       </c>
       <c r="H4" t="n">
-        <v>90.16000366210938</v>
+        <v>93.55999755859375</v>
       </c>
       <c r="I4" t="n">
-        <v>21.63</v>
+        <v>20.63</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -4203,14 +4203,14 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>bullish trend</t>
+          <t>bullish trend, potentially oversold</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SI=F</t>
+          <t>CL=F</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4219,7 +4219,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.7030999999999999</v>
+        <v>0.6949</v>
       </c>
       <c r="D5" t="n">
         <v>0.5</v>
@@ -4228,16 +4228,16 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>1.94</v>
+        <v>1.91</v>
       </c>
       <c r="G5" t="n">
-        <v>1940</v>
+        <v>1910</v>
       </c>
       <c r="H5" t="n">
-        <v>74.77999877929688</v>
+        <v>90.16000366210938</v>
       </c>
       <c r="I5" t="n">
-        <v>25.94</v>
+        <v>21.18</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -4256,7 +4256,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>^VIX</t>
+          <t>SI=F</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4265,7 +4265,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.6997</v>
+        <v>0.694</v>
       </c>
       <c r="D6" t="n">
         <v>0.5</v>
@@ -4274,16 +4274,16 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>1.93</v>
+        <v>1.91</v>
       </c>
       <c r="G6" t="n">
-        <v>1930</v>
+        <v>1910</v>
       </c>
       <c r="H6" t="n">
-        <v>16.95000076293945</v>
+        <v>74.77999877929688</v>
       </c>
       <c r="I6" t="n">
-        <v>113.86</v>
+        <v>25.54</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.6869</v>
+        <v>0.6825</v>
       </c>
       <c r="D7" t="n">
         <v>0.5</v>
@@ -4320,16 +4320,16 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>1.89</v>
+        <v>1.88</v>
       </c>
       <c r="G7" t="n">
-        <v>1890</v>
+        <v>1880</v>
       </c>
       <c r="H7" t="n">
         <v>6.335000038146973</v>
       </c>
       <c r="I7" t="n">
-        <v>298.34</v>
+        <v>296.76</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -4357,7 +4357,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.6712</v>
+        <v>0.6758</v>
       </c>
       <c r="D8" t="n">
         <v>0.5</v>
@@ -4366,16 +4366,16 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>1.84</v>
+        <v>1.86</v>
       </c>
       <c r="G8" t="n">
-        <v>1840</v>
+        <v>1860</v>
       </c>
       <c r="H8" t="n">
         <v>99.22200012207031</v>
       </c>
       <c r="I8" t="n">
-        <v>18.54</v>
+        <v>18.75</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -4403,7 +4403,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.3695</v>
+        <v>0.3676</v>
       </c>
       <c r="D9" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
achieved a stable point
</commit_message>
<xml_diff>
--- a/data/exports/dev-portfolio_intelligence.xlsx
+++ b/data/exports/dev-portfolio_intelligence.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="204">
   <si>
     <t>trade_date</t>
   </si>
@@ -518,7 +518,7 @@
     <t>potentially oversold</t>
   </si>
   <si>
-    <t>risk_score</t>
+    <t>asset_risk_score</t>
   </si>
   <si>
     <t>portfolio_risk</t>
@@ -549,6 +549,9 @@
   </si>
   <si>
     <t>tax_score</t>
+  </si>
+  <si>
+    <t>position_risk_score</t>
   </si>
   <si>
     <t>holding_score</t>
@@ -1486,13 +1489,13 @@
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1500,16 +1503,16 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D2">
         <v>3963.91</v>
       </c>
       <c r="E2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1517,16 +1520,16 @@
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D3">
         <v>2834.03</v>
       </c>
       <c r="E3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1534,16 +1537,16 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D4">
         <v>1228.97</v>
       </c>
       <c r="E4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -1564,10 +1567,10 @@
         <v>48</v>
       </c>
       <c r="C1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1581,7 +1584,7 @@
         <v>49.98</v>
       </c>
       <c r="D2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1595,7 +1598,7 @@
         <v>34.89</v>
       </c>
       <c r="D3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1609,7 +1612,7 @@
         <v>15.13</v>
       </c>
       <c r="D4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -1624,7 +1627,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
@@ -1644,7 +1647,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -1664,7 +1667,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B3" t="s">
         <v>17</v>
@@ -1684,7 +1687,7 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -1704,7 +1707,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
@@ -1724,7 +1727,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
@@ -1744,7 +1747,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -1764,7 +1767,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B8" t="s">
         <v>10</v>
@@ -1784,7 +1787,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B9" t="s">
         <v>17</v>
@@ -1804,7 +1807,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
@@ -1840,13 +1843,13 @@
         <v>3</v>
       </c>
       <c r="C1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D1" t="s">
         <v>179</v>
       </c>
-      <c r="D1" t="s">
-        <v>178</v>
-      </c>
       <c r="E1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1860,10 +1863,10 @@
         <v>3963.91</v>
       </c>
       <c r="D2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1877,10 +1880,10 @@
         <v>2834.03</v>
       </c>
       <c r="D3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1894,10 +1897,10 @@
         <v>1228.97</v>
       </c>
       <c r="D4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -1917,15 +1920,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B2">
         <v>40000</v>
@@ -1933,7 +1936,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B3">
         <v>15000</v>
@@ -1941,7 +1944,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B4">
         <v>20000</v>
@@ -1949,7 +1952,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B5">
         <v>12000</v>
@@ -1957,7 +1960,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B6">
         <v>33738.31</v>
@@ -1965,7 +1968,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B7">
         <v>70</v>
@@ -1973,7 +1976,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B8">
         <v>28000</v>
@@ -1981,7 +1984,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B9">
         <v>13000</v>
@@ -13344,10 +13347,10 @@
         <v>173</v>
       </c>
       <c r="H1" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="I1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J1" t="s">
         <v>154</v>
@@ -13382,7 +13385,7 @@
         <v>0.8892</v>
       </c>
       <c r="J2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -13414,7 +13417,7 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -13446,7 +13449,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
good stable point with unit and integration test
</commit_message>
<xml_diff>
--- a/data/exports/dev-portfolio_intelligence.xlsx
+++ b/data/exports/dev-portfolio_intelligence.xlsx
@@ -629,7 +629,7 @@
     <t>TargetCashReserve</t>
   </si>
   <si>
-    <t>MonthlyContributions</t>
+    <t>Contributions</t>
   </si>
   <si>
     <t>MaxDeploymentPercent</t>
@@ -11843,7 +11843,7 @@
         <v>0.4085</v>
       </c>
       <c r="D41">
-        <v>0.3076</v>
+        <v>0.3085</v>
       </c>
       <c r="E41">
         <v>0</v>

</xml_diff>

<commit_message>
Drive sell pipeline from capital state
</commit_message>
<xml_diff>
--- a/data/exports/dev-portfolio_intelligence.xlsx
+++ b/data/exports/dev-portfolio_intelligence.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1243" uniqueCount="216">
   <si>
     <t>trade_date</t>
   </si>
@@ -617,28 +617,64 @@
     <t>Value</t>
   </si>
   <si>
-    <t>PortfolioValue</t>
-  </si>
-  <si>
-    <t>CurrentCash</t>
-  </si>
-  <si>
-    <t>EmergencyReserve</t>
-  </si>
-  <si>
-    <t>TargetCashReserve</t>
-  </si>
-  <si>
-    <t>Contributions</t>
-  </si>
-  <si>
-    <t>MaxDeploymentPercent</t>
-  </si>
-  <si>
-    <t>DeployableCapital</t>
-  </si>
-  <si>
-    <t>AvailableToInvest</t>
+    <t>cash</t>
+  </si>
+  <si>
+    <t>target_cash_reserve</t>
+  </si>
+  <si>
+    <t>cash_shortfall</t>
+  </si>
+  <si>
+    <t>cash_surplus</t>
+  </si>
+  <si>
+    <t>portfolio_value</t>
+  </si>
+  <si>
+    <t>invested_value</t>
+  </si>
+  <si>
+    <t>max_deployment_percent</t>
+  </si>
+  <si>
+    <t>target_invested_value</t>
+  </si>
+  <si>
+    <t>deployment_difference</t>
+  </si>
+  <si>
+    <t>required_sale_value</t>
+  </si>
+  <si>
+    <t>available_cash</t>
+  </si>
+  <si>
+    <t>deployable_capital</t>
+  </si>
+  <si>
+    <t>required_sale_for_cash</t>
+  </si>
+  <si>
+    <t>required_sale_for_deployment</t>
+  </si>
+  <si>
+    <t>cash_target_achievable</t>
+  </si>
+  <si>
+    <t>capital_status</t>
+  </si>
+  <si>
+    <t>cash_funding_ratio</t>
+  </si>
+  <si>
+    <t>cash_percentage</t>
+  </si>
+  <si>
+    <t>invested_percentage</t>
+  </si>
+  <si>
+    <t>CRITICAL</t>
   </si>
 </sst>
 </file>
@@ -1509,7 +1545,7 @@
         <v>183</v>
       </c>
       <c r="D2">
-        <v>3820.98</v>
+        <v>3815.2</v>
       </c>
       <c r="E2" t="s">
         <v>185</v>
@@ -1526,7 +1562,7 @@
         <v>183</v>
       </c>
       <c r="D3">
-        <v>2730.88</v>
+        <v>2741.29</v>
       </c>
       <c r="E3" t="s">
         <v>185</v>
@@ -1543,7 +1579,7 @@
         <v>184</v>
       </c>
       <c r="D4">
-        <v>1389.16</v>
+        <v>1418.69</v>
       </c>
       <c r="E4" t="s">
         <v>186</v>
@@ -1578,10 +1614,10 @@
         <v>149</v>
       </c>
       <c r="B2">
-        <v>3918.9</v>
+        <v>3915.9</v>
       </c>
       <c r="C2">
-        <v>48.75</v>
+        <v>48.49</v>
       </c>
       <c r="D2" t="s">
         <v>183</v>
@@ -1592,10 +1628,10 @@
         <v>148</v>
       </c>
       <c r="B3">
-        <v>2731.2</v>
+        <v>2741.4</v>
       </c>
       <c r="C3">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="D3" t="s">
         <v>184</v>
@@ -1606,10 +1642,10 @@
         <v>147</v>
       </c>
       <c r="B4">
-        <v>1389</v>
+        <v>1418</v>
       </c>
       <c r="C4">
-        <v>17.28</v>
+        <v>17.56</v>
       </c>
       <c r="D4" t="s">
         <v>189</v>
@@ -1656,13 +1692,13 @@
         <v>100</v>
       </c>
       <c r="D2">
-        <v>1389</v>
+        <v>1418</v>
       </c>
       <c r="E2">
-        <v>836</v>
+        <v>865</v>
       </c>
       <c r="F2">
-        <v>1.0279</v>
+        <v>1.0267</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1676,13 +1712,13 @@
         <v>60</v>
       </c>
       <c r="D3">
-        <v>2731.2</v>
+        <v>2741.4</v>
       </c>
       <c r="E3">
-        <v>2281.2</v>
+        <v>2291.4</v>
       </c>
       <c r="F3">
-        <v>0.8260999999999999</v>
+        <v>0.8206</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1693,16 +1729,16 @@
         <v>14</v>
       </c>
       <c r="C4">
-        <v>3.37</v>
+        <v>3.22</v>
       </c>
       <c r="D4">
-        <v>879.8</v>
+        <v>840.6</v>
       </c>
       <c r="E4">
-        <v>454.14</v>
+        <v>433.6</v>
       </c>
       <c r="F4">
-        <v>0.4572</v>
+        <v>0.4547</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1716,13 +1752,13 @@
         <v>100</v>
       </c>
       <c r="D5">
-        <v>1389</v>
+        <v>1418</v>
       </c>
       <c r="E5">
-        <v>836</v>
+        <v>865</v>
       </c>
       <c r="F5">
-        <v>0.9835</v>
+        <v>0.9824000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1736,13 +1772,13 @@
         <v>60</v>
       </c>
       <c r="D6">
-        <v>2731.2</v>
+        <v>2741.4</v>
       </c>
       <c r="E6">
-        <v>2281.2</v>
+        <v>2291.4</v>
       </c>
       <c r="F6">
-        <v>0.9199000000000001</v>
+        <v>0.9144</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1753,16 +1789,16 @@
         <v>14</v>
       </c>
       <c r="C7">
-        <v>3.37</v>
+        <v>3.22</v>
       </c>
       <c r="D7">
-        <v>879.8</v>
+        <v>840.6</v>
       </c>
       <c r="E7">
-        <v>454.14</v>
+        <v>433.6</v>
       </c>
       <c r="F7">
-        <v>0.4572</v>
+        <v>0.4547</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1776,13 +1812,13 @@
         <v>100</v>
       </c>
       <c r="D8">
-        <v>1389</v>
+        <v>1418</v>
       </c>
       <c r="E8">
-        <v>836</v>
+        <v>865</v>
       </c>
       <c r="F8">
-        <v>0.6279</v>
+        <v>0.6267</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1796,13 +1832,13 @@
         <v>60</v>
       </c>
       <c r="D9">
-        <v>2731.2</v>
+        <v>2741.4</v>
       </c>
       <c r="E9">
-        <v>2281.2</v>
+        <v>2291.4</v>
       </c>
       <c r="F9">
-        <v>0.7321</v>
+        <v>0.7262999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1813,16 +1849,16 @@
         <v>14</v>
       </c>
       <c r="C10">
-        <v>3.37</v>
+        <v>3.22</v>
       </c>
       <c r="D10">
-        <v>879.8</v>
+        <v>840.6</v>
       </c>
       <c r="E10">
-        <v>454.14</v>
+        <v>433.6</v>
       </c>
       <c r="F10">
-        <v>0.8572</v>
+        <v>0.8547</v>
       </c>
     </row>
   </sheetData>
@@ -1860,7 +1896,7 @@
         <v>19</v>
       </c>
       <c r="C2">
-        <v>3820.98</v>
+        <v>3815.2</v>
       </c>
       <c r="D2" t="s">
         <v>183</v>
@@ -1877,7 +1913,7 @@
         <v>19</v>
       </c>
       <c r="C3">
-        <v>2730.88</v>
+        <v>2741.29</v>
       </c>
       <c r="D3" t="s">
         <v>183</v>
@@ -1894,7 +1930,7 @@
         <v>19</v>
       </c>
       <c r="C4">
-        <v>1389.16</v>
+        <v>1418.69</v>
       </c>
       <c r="D4" t="s">
         <v>184</v>
@@ -1910,7 +1946,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1931,7 +1967,7 @@
         <v>196</v>
       </c>
       <c r="B2">
-        <v>40000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1939,7 +1975,7 @@
         <v>197</v>
       </c>
       <c r="B3">
-        <v>15000</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1947,7 +1983,7 @@
         <v>198</v>
       </c>
       <c r="B4">
-        <v>20000</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1955,7 +1991,7 @@
         <v>199</v>
       </c>
       <c r="B5">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1963,7 +1999,7 @@
         <v>200</v>
       </c>
       <c r="B6">
-        <v>1000</v>
+        <v>8076.62</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1971,7 +2007,7 @@
         <v>201</v>
       </c>
       <c r="B7">
-        <v>50</v>
+        <v>8076.62</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1979,7 +2015,7 @@
         <v>202</v>
       </c>
       <c r="B8">
-        <v>20000</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1987,7 +2023,95 @@
         <v>203</v>
       </c>
       <c r="B9">
-        <v>5000</v>
+        <v>5653.63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>204</v>
+      </c>
+      <c r="B10">
+        <v>2422.99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>205</v>
+      </c>
+      <c r="B11">
+        <v>2422.99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>206</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>207</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>208</v>
+      </c>
+      <c r="B14">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>209</v>
+      </c>
+      <c r="B15">
+        <v>2422.99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>210</v>
+      </c>
+      <c r="B16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>211</v>
+      </c>
+      <c r="B17" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>212</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>213</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>214</v>
+      </c>
+      <c r="B20">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2614,7 +2738,7 @@
         <v>34</v>
       </c>
       <c r="K2">
-        <v>13.89</v>
+        <v>14.18</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -2658,19 +2782,19 @@
         <v>553</v>
       </c>
       <c r="K3">
-        <v>13.89</v>
+        <v>14.18</v>
       </c>
       <c r="L3">
-        <v>1389</v>
+        <v>1418</v>
       </c>
       <c r="M3">
         <v>553</v>
       </c>
       <c r="N3">
-        <v>836</v>
+        <v>865</v>
       </c>
       <c r="O3">
-        <v>151.18</v>
+        <v>156.42</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -2705,7 +2829,7 @@
         <v>32</v>
       </c>
       <c r="K4">
-        <v>600.47</v>
+        <v>607.37</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -2752,7 +2876,7 @@
         <v>33</v>
       </c>
       <c r="K5">
-        <v>224.36</v>
+        <v>225.99</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -2799,7 +2923,7 @@
         <v>34</v>
       </c>
       <c r="K6">
-        <v>415.88</v>
+        <v>422.15</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -2846,19 +2970,19 @@
         <v>34</v>
       </c>
       <c r="K7">
-        <v>261.26</v>
+        <v>261.06</v>
       </c>
       <c r="L7">
-        <v>3918.9</v>
+        <v>3915.9</v>
       </c>
       <c r="M7">
         <v>1896</v>
       </c>
       <c r="N7">
-        <v>2022.9</v>
+        <v>2019.9</v>
       </c>
       <c r="O7">
-        <v>106.69</v>
+        <v>106.53</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -2893,7 +3017,7 @@
         <v>34</v>
       </c>
       <c r="K8">
-        <v>372.58</v>
+        <v>366.7</v>
       </c>
       <c r="L8">
         <v>0</v>
@@ -2940,7 +3064,7 @@
         <v>34</v>
       </c>
       <c r="K9">
-        <v>160.65</v>
+        <v>150.9</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -2987,19 +3111,19 @@
         <v>34</v>
       </c>
       <c r="K10">
-        <v>45.52</v>
+        <v>45.69</v>
       </c>
       <c r="L10">
-        <v>2731.2</v>
+        <v>2741.4</v>
       </c>
       <c r="M10">
         <v>450</v>
       </c>
       <c r="N10">
-        <v>2281.2</v>
+        <v>2291.4</v>
       </c>
       <c r="O10">
-        <v>506.93</v>
+        <v>509.2</v>
       </c>
     </row>
   </sheetData>
@@ -3265,7 +3389,7 @@
         <v>0.7016</v>
       </c>
       <c r="J5">
-        <v>0.8011</v>
+        <v>0.8007</v>
       </c>
       <c r="K5" t="s">
         <v>142</v>
@@ -3274,10 +3398,10 @@
         <v>147</v>
       </c>
       <c r="M5">
-        <v>17.28</v>
+        <v>17.57</v>
       </c>
       <c r="N5">
-        <v>0.8272</v>
+        <v>0.8243</v>
       </c>
       <c r="O5" t="s">
         <v>153</v>
@@ -3321,7 +3445,7 @@
         <v>0.4721</v>
       </c>
       <c r="J6">
-        <v>0.7638</v>
+        <v>0.7634</v>
       </c>
       <c r="K6" t="s">
         <v>18</v>
@@ -3330,10 +3454,10 @@
         <v>147</v>
       </c>
       <c r="M6">
-        <v>17.28</v>
+        <v>17.57</v>
       </c>
       <c r="N6">
-        <v>0.8272</v>
+        <v>0.8243</v>
       </c>
       <c r="O6" t="s">
         <v>153</v>
@@ -3386,10 +3510,10 @@
         <v>148</v>
       </c>
       <c r="M7">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N7">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O7" t="s">
         <v>153</v>
@@ -3442,10 +3566,10 @@
         <v>148</v>
       </c>
       <c r="M8">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N8">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O8" t="s">
         <v>153</v>
@@ -3498,10 +3622,10 @@
         <v>148</v>
       </c>
       <c r="M9">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N9">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O9" t="s">
         <v>153</v>
@@ -3554,10 +3678,10 @@
         <v>148</v>
       </c>
       <c r="M10">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N10">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O10" t="s">
         <v>153</v>
@@ -3610,10 +3734,10 @@
         <v>148</v>
       </c>
       <c r="M11">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N11">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O11" t="s">
         <v>153</v>
@@ -3666,10 +3790,10 @@
         <v>148</v>
       </c>
       <c r="M12">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N12">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O12" t="s">
         <v>153</v>
@@ -3722,10 +3846,10 @@
         <v>148</v>
       </c>
       <c r="M13">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N13">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O13" t="s">
         <v>153</v>
@@ -3769,7 +3893,7 @@
         <v>0.4798</v>
       </c>
       <c r="J14">
-        <v>0.6749000000000001</v>
+        <v>0.675</v>
       </c>
       <c r="K14" t="s">
         <v>18</v>
@@ -3778,10 +3902,10 @@
         <v>148</v>
       </c>
       <c r="M14">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N14">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O14" t="s">
         <v>153</v>
@@ -3834,10 +3958,10 @@
         <v>148</v>
       </c>
       <c r="M15">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N15">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O15" t="s">
         <v>153</v>
@@ -3890,10 +4014,10 @@
         <v>148</v>
       </c>
       <c r="M16">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N16">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O16" t="s">
         <v>153</v>
@@ -3946,10 +4070,10 @@
         <v>148</v>
       </c>
       <c r="M17">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N17">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O17" t="s">
         <v>153</v>
@@ -4002,10 +4126,10 @@
         <v>148</v>
       </c>
       <c r="M18">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N18">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O18" t="s">
         <v>153</v>
@@ -4049,7 +4173,7 @@
         <v>0.4626</v>
       </c>
       <c r="J19">
-        <v>0.6627</v>
+        <v>0.6627999999999999</v>
       </c>
       <c r="K19" t="s">
         <v>18</v>
@@ -4058,10 +4182,10 @@
         <v>148</v>
       </c>
       <c r="M19">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N19">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O19" t="s">
         <v>153</v>
@@ -4114,10 +4238,10 @@
         <v>148</v>
       </c>
       <c r="M20">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N20">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O20" t="s">
         <v>153</v>
@@ -4161,7 +4285,7 @@
         <v>0.4511</v>
       </c>
       <c r="J21">
-        <v>0.6621</v>
+        <v>0.6622</v>
       </c>
       <c r="K21" t="s">
         <v>18</v>
@@ -4170,10 +4294,10 @@
         <v>148</v>
       </c>
       <c r="M21">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N21">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O21" t="s">
         <v>153</v>
@@ -4217,7 +4341,7 @@
         <v>0.3831</v>
       </c>
       <c r="J22">
-        <v>0.6616</v>
+        <v>0.6617</v>
       </c>
       <c r="K22" t="s">
         <v>18</v>
@@ -4226,10 +4350,10 @@
         <v>148</v>
       </c>
       <c r="M22">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N22">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O22" t="s">
         <v>153</v>
@@ -4273,7 +4397,7 @@
         <v>0.5249</v>
       </c>
       <c r="J23">
-        <v>0.6529</v>
+        <v>0.6533</v>
       </c>
       <c r="K23" t="s">
         <v>18</v>
@@ -4282,10 +4406,10 @@
         <v>149</v>
       </c>
       <c r="M23">
-        <v>48.75</v>
+        <v>48.48</v>
       </c>
       <c r="N23">
-        <v>0.5125</v>
+        <v>0.5152</v>
       </c>
       <c r="O23" t="s">
         <v>153</v>
@@ -4329,7 +4453,7 @@
         <v>0.4292</v>
       </c>
       <c r="J24">
-        <v>0.6524</v>
+        <v>0.6525</v>
       </c>
       <c r="K24" t="s">
         <v>18</v>
@@ -4338,10 +4462,10 @@
         <v>148</v>
       </c>
       <c r="M24">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N24">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O24" t="s">
         <v>153</v>
@@ -4385,7 +4509,7 @@
         <v>0.3639</v>
       </c>
       <c r="J25">
-        <v>0.6509</v>
+        <v>0.651</v>
       </c>
       <c r="K25" t="s">
         <v>18</v>
@@ -4394,10 +4518,10 @@
         <v>148</v>
       </c>
       <c r="M25">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N25">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O25" t="s">
         <v>153</v>
@@ -4450,10 +4574,10 @@
         <v>148</v>
       </c>
       <c r="M26">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N26">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O26" t="s">
         <v>153</v>
@@ -4497,7 +4621,7 @@
         <v>0.3322</v>
       </c>
       <c r="J27">
-        <v>0.649</v>
+        <v>0.6491</v>
       </c>
       <c r="K27" t="s">
         <v>18</v>
@@ -4506,10 +4630,10 @@
         <v>148</v>
       </c>
       <c r="M27">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N27">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O27" t="s">
         <v>153</v>
@@ -4553,7 +4677,7 @@
         <v>0.3869</v>
       </c>
       <c r="J28">
-        <v>0.6448</v>
+        <v>0.6449</v>
       </c>
       <c r="K28" t="s">
         <v>18</v>
@@ -4562,10 +4686,10 @@
         <v>148</v>
       </c>
       <c r="M28">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N28">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O28" t="s">
         <v>153</v>
@@ -4618,10 +4742,10 @@
         <v>148</v>
       </c>
       <c r="M29">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N29">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O29" t="s">
         <v>153</v>
@@ -4674,10 +4798,10 @@
         <v>148</v>
       </c>
       <c r="M30">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N30">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O30" t="s">
         <v>153</v>
@@ -4730,10 +4854,10 @@
         <v>148</v>
       </c>
       <c r="M31">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N31">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O31" t="s">
         <v>153</v>
@@ -4786,10 +4910,10 @@
         <v>148</v>
       </c>
       <c r="M32">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N32">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O32" t="s">
         <v>153</v>
@@ -4842,10 +4966,10 @@
         <v>148</v>
       </c>
       <c r="M33">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N33">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O33" t="s">
         <v>153</v>
@@ -4898,10 +5022,10 @@
         <v>148</v>
       </c>
       <c r="M34">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N34">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O34" t="s">
         <v>153</v>
@@ -4954,10 +5078,10 @@
         <v>148</v>
       </c>
       <c r="M35">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N35">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O35" t="s">
         <v>153</v>
@@ -5010,10 +5134,10 @@
         <v>148</v>
       </c>
       <c r="M36">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N36">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O36" t="s">
         <v>153</v>
@@ -5066,10 +5190,10 @@
         <v>148</v>
       </c>
       <c r="M37">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N37">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O37" t="s">
         <v>153</v>
@@ -5122,10 +5246,10 @@
         <v>148</v>
       </c>
       <c r="M38">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N38">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O38" t="s">
         <v>153</v>
@@ -5169,7 +5293,7 @@
         <v>0.177</v>
       </c>
       <c r="J39">
-        <v>0.6253</v>
+        <v>0.6254</v>
       </c>
       <c r="K39" t="s">
         <v>18</v>
@@ -5178,10 +5302,10 @@
         <v>148</v>
       </c>
       <c r="M39">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N39">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O39" t="s">
         <v>153</v>
@@ -5234,10 +5358,10 @@
         <v>148</v>
       </c>
       <c r="M40">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N40">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O40" t="s">
         <v>153</v>
@@ -5290,10 +5414,10 @@
         <v>148</v>
       </c>
       <c r="M41">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N41">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O41" t="s">
         <v>153</v>
@@ -5346,10 +5470,10 @@
         <v>148</v>
       </c>
       <c r="M42">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N42">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O42" t="s">
         <v>153</v>
@@ -5393,7 +5517,7 @@
         <v>0.1524</v>
       </c>
       <c r="J43">
-        <v>0.6236</v>
+        <v>0.6237</v>
       </c>
       <c r="K43" t="s">
         <v>18</v>
@@ -5402,10 +5526,10 @@
         <v>148</v>
       </c>
       <c r="M43">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N43">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O43" t="s">
         <v>153</v>
@@ -5449,7 +5573,7 @@
         <v>0.1162</v>
       </c>
       <c r="J44">
-        <v>0.6127</v>
+        <v>0.6128</v>
       </c>
       <c r="K44" t="s">
         <v>18</v>
@@ -5458,10 +5582,10 @@
         <v>148</v>
       </c>
       <c r="M44">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N44">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O44" t="s">
         <v>153</v>
@@ -5626,10 +5750,10 @@
         <v>148</v>
       </c>
       <c r="M47">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N47">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O47" t="s">
         <v>153</v>
@@ -5738,10 +5862,10 @@
         <v>148</v>
       </c>
       <c r="M49">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N49">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O49" t="s">
         <v>153</v>
@@ -5794,10 +5918,10 @@
         <v>148</v>
       </c>
       <c r="M50">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N50">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O50" t="s">
         <v>153</v>
@@ -5850,10 +5974,10 @@
         <v>148</v>
       </c>
       <c r="M51">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N51">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O51" t="s">
         <v>153</v>
@@ -5906,10 +6030,10 @@
         <v>148</v>
       </c>
       <c r="M52">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N52">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O52" t="s">
         <v>153</v>
@@ -5962,10 +6086,10 @@
         <v>148</v>
       </c>
       <c r="M53">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N53">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O53" t="s">
         <v>153</v>
@@ -6018,10 +6142,10 @@
         <v>148</v>
       </c>
       <c r="M54">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N54">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O54" t="s">
         <v>153</v>
@@ -6074,10 +6198,10 @@
         <v>148</v>
       </c>
       <c r="M55">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N55">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O55" t="s">
         <v>153</v>
@@ -6130,10 +6254,10 @@
         <v>148</v>
       </c>
       <c r="M56">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N56">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O56" t="s">
         <v>153</v>
@@ -6186,10 +6310,10 @@
         <v>148</v>
       </c>
       <c r="M57">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N57">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O57" t="s">
         <v>153</v>
@@ -6233,7 +6357,7 @@
         <v>0.4911</v>
       </c>
       <c r="J58">
-        <v>0.372</v>
+        <v>0.3721</v>
       </c>
       <c r="K58" t="s">
         <v>144</v>
@@ -6242,10 +6366,10 @@
         <v>148</v>
       </c>
       <c r="M58">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N58">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O58" t="s">
         <v>153</v>
@@ -6298,10 +6422,10 @@
         <v>148</v>
       </c>
       <c r="M59">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N59">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O59" t="s">
         <v>153</v>
@@ -6354,10 +6478,10 @@
         <v>148</v>
       </c>
       <c r="M60">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N60">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O60" t="s">
         <v>153</v>
@@ -6410,10 +6534,10 @@
         <v>148</v>
       </c>
       <c r="M61">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N61">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O61" t="s">
         <v>153</v>
@@ -6466,10 +6590,10 @@
         <v>148</v>
       </c>
       <c r="M62">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N62">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O62" t="s">
         <v>153</v>
@@ -6522,10 +6646,10 @@
         <v>148</v>
       </c>
       <c r="M63">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N63">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O63" t="s">
         <v>153</v>
@@ -6578,10 +6702,10 @@
         <v>148</v>
       </c>
       <c r="M64">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N64">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O64" t="s">
         <v>153</v>
@@ -6634,10 +6758,10 @@
         <v>148</v>
       </c>
       <c r="M65">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N65">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O65" t="s">
         <v>153</v>
@@ -6690,10 +6814,10 @@
         <v>148</v>
       </c>
       <c r="M66">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N66">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O66" t="s">
         <v>153</v>
@@ -6746,10 +6870,10 @@
         <v>148</v>
       </c>
       <c r="M67">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N67">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O67" t="s">
         <v>153</v>
@@ -6802,10 +6926,10 @@
         <v>148</v>
       </c>
       <c r="M68">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N68">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O68" t="s">
         <v>153</v>
@@ -6849,7 +6973,7 @@
         <v>0.3708</v>
       </c>
       <c r="J69">
-        <v>0.3527</v>
+        <v>0.3528</v>
       </c>
       <c r="K69" t="s">
         <v>144</v>
@@ -6858,10 +6982,10 @@
         <v>148</v>
       </c>
       <c r="M69">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N69">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O69" t="s">
         <v>153</v>
@@ -6914,10 +7038,10 @@
         <v>148</v>
       </c>
       <c r="M70">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N70">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O70" t="s">
         <v>153</v>
@@ -6961,7 +7085,7 @@
         <v>0.3412</v>
       </c>
       <c r="J71">
-        <v>0.3495</v>
+        <v>0.3496</v>
       </c>
       <c r="K71" t="s">
         <v>144</v>
@@ -6970,10 +7094,10 @@
         <v>148</v>
       </c>
       <c r="M71">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N71">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O71" t="s">
         <v>153</v>
@@ -7026,10 +7150,10 @@
         <v>148</v>
       </c>
       <c r="M72">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N72">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O72" t="s">
         <v>153</v>
@@ -7082,10 +7206,10 @@
         <v>148</v>
       </c>
       <c r="M73">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N73">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O73" t="s">
         <v>153</v>
@@ -7138,10 +7262,10 @@
         <v>148</v>
       </c>
       <c r="M74">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N74">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O74" t="s">
         <v>153</v>
@@ -7185,7 +7309,7 @@
         <v>0.2727</v>
       </c>
       <c r="J75">
-        <v>0.3407</v>
+        <v>0.3408</v>
       </c>
       <c r="K75" t="s">
         <v>144</v>
@@ -7194,10 +7318,10 @@
         <v>148</v>
       </c>
       <c r="M75">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N75">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O75" t="s">
         <v>153</v>
@@ -7250,10 +7374,10 @@
         <v>148</v>
       </c>
       <c r="M76">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N76">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O76" t="s">
         <v>153</v>
@@ -7306,10 +7430,10 @@
         <v>148</v>
       </c>
       <c r="M77">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N77">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O77" t="s">
         <v>153</v>
@@ -7362,10 +7486,10 @@
         <v>148</v>
       </c>
       <c r="M78">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N78">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O78" t="s">
         <v>153</v>
@@ -7418,10 +7542,10 @@
         <v>148</v>
       </c>
       <c r="M79">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N79">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O79" t="s">
         <v>153</v>
@@ -7474,10 +7598,10 @@
         <v>148</v>
       </c>
       <c r="M80">
-        <v>33.97</v>
+        <v>33.95</v>
       </c>
       <c r="N80">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="O80" t="s">
         <v>153</v>
@@ -7653,7 +7777,7 @@
         <v>10.6201000213623</v>
       </c>
       <c r="D5">
-        <v>0.8011</v>
+        <v>0.8007</v>
       </c>
       <c r="E5">
         <v>11.68120206832886</v>
@@ -7671,7 +7795,7 @@
         <v>29.84059297913404</v>
       </c>
       <c r="J5">
-        <v>0.8272</v>
+        <v>0.8243</v>
       </c>
       <c r="K5" t="s">
         <v>157</v>
@@ -7688,7 +7812,7 @@
         <v>12.17000007629395</v>
       </c>
       <c r="D6">
-        <v>0.7638</v>
+        <v>0.7634</v>
       </c>
       <c r="E6">
         <v>9.490199975967407</v>
@@ -7706,7 +7830,7 @@
         <v>52.79048555853054</v>
       </c>
       <c r="J6">
-        <v>0.8272</v>
+        <v>0.8243</v>
       </c>
       <c r="K6" t="s">
         <v>156</v>
@@ -7741,7 +7865,7 @@
         <v>24.32237410558415</v>
       </c>
       <c r="J7">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K7" t="s">
         <v>158</v>
@@ -7776,7 +7900,7 @@
         <v>34.93956665818956</v>
       </c>
       <c r="J8">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K8" t="s">
         <v>158</v>
@@ -7811,7 +7935,7 @@
         <v>55.74873620999067</v>
       </c>
       <c r="J9">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K9" t="s">
         <v>159</v>
@@ -7846,7 +7970,7 @@
         <v>42.79099330023248</v>
       </c>
       <c r="J10">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K10" t="s">
         <v>159</v>
@@ -7881,7 +8005,7 @@
         <v>39.25098385656076</v>
       </c>
       <c r="J11">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K11" t="s">
         <v>158</v>
@@ -7916,7 +8040,7 @@
         <v>41.29244115486681</v>
       </c>
       <c r="J12">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K12" t="s">
         <v>159</v>
@@ -7951,7 +8075,7 @@
         <v>47.29547809343844</v>
       </c>
       <c r="J13">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K13" t="s">
         <v>159</v>
@@ -7968,7 +8092,7 @@
         <v>156.1300048828125</v>
       </c>
       <c r="D14">
-        <v>0.6749000000000001</v>
+        <v>0.675</v>
       </c>
       <c r="E14">
         <v>147.9280003356934</v>
@@ -7986,7 +8110,7 @@
         <v>52.01954969224415</v>
       </c>
       <c r="J14">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K14" t="s">
         <v>159</v>
@@ -8021,7 +8145,7 @@
         <v>50.0953380320746</v>
       </c>
       <c r="J15">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K15" t="s">
         <v>159</v>
@@ -8056,7 +8180,7 @@
         <v>49.58712417755017</v>
       </c>
       <c r="J16">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K16" t="s">
         <v>159</v>
@@ -8091,7 +8215,7 @@
         <v>55.81680137154054</v>
       </c>
       <c r="J17">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K17" t="s">
         <v>159</v>
@@ -8126,7 +8250,7 @@
         <v>52.52196685210854</v>
       </c>
       <c r="J18">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K18" t="s">
         <v>159</v>
@@ -8143,7 +8267,7 @@
         <v>437.3999938964844</v>
       </c>
       <c r="D19">
-        <v>0.6627</v>
+        <v>0.6627999999999999</v>
       </c>
       <c r="E19">
         <v>385.4850103759766</v>
@@ -8161,7 +8285,7 @@
         <v>53.74493548838463</v>
       </c>
       <c r="J19">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K19" t="s">
         <v>159</v>
@@ -8196,7 +8320,7 @@
         <v>53.33591079169458</v>
       </c>
       <c r="J20">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K20" t="s">
         <v>159</v>
@@ -8213,7 +8337,7 @@
         <v>1930.010009765625</v>
       </c>
       <c r="D21">
-        <v>0.6621</v>
+        <v>0.6622</v>
       </c>
       <c r="E21">
         <v>1730.606733398437</v>
@@ -8231,7 +8355,7 @@
         <v>54.89072413854991</v>
       </c>
       <c r="J21">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K21" t="s">
         <v>159</v>
@@ -8248,7 +8372,7 @@
         <v>104.2600021362305</v>
       </c>
       <c r="D22">
-        <v>0.6616</v>
+        <v>0.6617</v>
       </c>
       <c r="E22">
         <v>57.82180000305176</v>
@@ -8266,7 +8390,7 @@
         <v>61.68698087643116</v>
       </c>
       <c r="J22">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K22" t="s">
         <v>159</v>
@@ -8283,7 +8407,7 @@
         <v>270.2804870605469</v>
       </c>
       <c r="D23">
-        <v>0.6529</v>
+        <v>0.6533</v>
       </c>
       <c r="E23">
         <v>246.6624099731445</v>
@@ -8301,7 +8425,7 @@
         <v>47.50671781742124</v>
       </c>
       <c r="J23">
-        <v>0.5125</v>
+        <v>0.5152</v>
       </c>
       <c r="K23" t="s">
         <v>159</v>
@@ -8318,7 +8442,7 @@
         <v>289.6799926757812</v>
       </c>
       <c r="D24">
-        <v>0.6524</v>
+        <v>0.6525</v>
       </c>
       <c r="E24">
         <v>270.0206011962891</v>
@@ -8336,7 +8460,7 @@
         <v>57.0804147127497</v>
       </c>
       <c r="J24">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K24" t="s">
         <v>159</v>
@@ -8353,7 +8477,7 @@
         <v>229.1600036621094</v>
       </c>
       <c r="D25">
-        <v>0.6509</v>
+        <v>0.651</v>
       </c>
       <c r="E25">
         <v>158.9171002197266</v>
@@ -8371,7 +8495,7 @@
         <v>63.60836779223327</v>
       </c>
       <c r="J25">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K25" t="s">
         <v>159</v>
@@ -8406,7 +8530,7 @@
         <v>72.55699795767705</v>
       </c>
       <c r="J26">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K26" t="s">
         <v>159</v>
@@ -8423,7 +8547,7 @@
         <v>160.1600036621094</v>
       </c>
       <c r="D27">
-        <v>0.649</v>
+        <v>0.6491</v>
       </c>
       <c r="E27">
         <v>148.8601998901367</v>
@@ -8441,7 +8565,7 @@
         <v>66.77614060250662</v>
       </c>
       <c r="J27">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K27" t="s">
         <v>159</v>
@@ -8458,7 +8582,7 @@
         <v>599.510009765625</v>
       </c>
       <c r="D28">
-        <v>0.6448</v>
+        <v>0.6449</v>
       </c>
       <c r="E28">
         <v>484.7420007324219</v>
@@ -8476,7 +8600,7 @@
         <v>61.30891593465972</v>
       </c>
       <c r="J28">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K28" t="s">
         <v>159</v>
@@ -8511,7 +8635,7 @@
         <v>68.00380242260704</v>
       </c>
       <c r="J29">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K29" t="s">
         <v>159</v>
@@ -8546,7 +8670,7 @@
         <v>68.7262179373717</v>
       </c>
       <c r="J30">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K30" t="s">
         <v>159</v>
@@ -8581,7 +8705,7 @@
         <v>73.3756782876756</v>
       </c>
       <c r="J31">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K31" t="s">
         <v>159</v>
@@ -8616,7 +8740,7 @@
         <v>63.72471183466363</v>
       </c>
       <c r="J32">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K32" t="s">
         <v>159</v>
@@ -8651,7 +8775,7 @@
         <v>75.71506554383619</v>
       </c>
       <c r="J33">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K33" t="s">
         <v>159</v>
@@ -8686,7 +8810,7 @@
         <v>79.18690654428941</v>
       </c>
       <c r="J34">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K34" t="s">
         <v>159</v>
@@ -8721,7 +8845,7 @@
         <v>67.11149544232157</v>
       </c>
       <c r="J35">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K35" t="s">
         <v>159</v>
@@ -8756,7 +8880,7 @@
         <v>68.69012892264033</v>
       </c>
       <c r="J36">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K36" t="s">
         <v>159</v>
@@ -8791,7 +8915,7 @@
         <v>80.7508215679068</v>
       </c>
       <c r="J37">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K37" t="s">
         <v>159</v>
@@ -8826,7 +8950,7 @@
         <v>84.59564438781432</v>
       </c>
       <c r="J38">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K38" t="s">
         <v>159</v>
@@ -8843,7 +8967,7 @@
         <v>279.1600036621094</v>
       </c>
       <c r="D39">
-        <v>0.6253</v>
+        <v>0.6254</v>
       </c>
       <c r="E39">
         <v>191.3692004394531</v>
@@ -8861,7 +8985,7 @@
         <v>82.30017258450833</v>
       </c>
       <c r="J39">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K39" t="s">
         <v>159</v>
@@ -8896,7 +9020,7 @@
         <v>83.40800204702586</v>
       </c>
       <c r="J40">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K40" t="s">
         <v>159</v>
@@ -8931,7 +9055,7 @@
         <v>80.72804757289227</v>
       </c>
       <c r="J41">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K41" t="s">
         <v>159</v>
@@ -8966,7 +9090,7 @@
         <v>82.2306288932008</v>
       </c>
       <c r="J42">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K42" t="s">
         <v>159</v>
@@ -8983,7 +9107,7 @@
         <v>416.2999877929688</v>
       </c>
       <c r="D43">
-        <v>0.6236</v>
+        <v>0.6237</v>
       </c>
       <c r="E43">
         <v>215.5247280883789</v>
@@ -9001,7 +9125,7 @@
         <v>84.76398843833833</v>
       </c>
       <c r="J43">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K43" t="s">
         <v>159</v>
@@ -9018,7 +9142,7 @@
         <v>726.155029296875</v>
       </c>
       <c r="D44">
-        <v>0.6127</v>
+        <v>0.6128</v>
       </c>
       <c r="E44">
         <v>482.4160998535156</v>
@@ -9036,7 +9160,7 @@
         <v>88.38347146788549</v>
       </c>
       <c r="J44">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K44" t="s">
         <v>159</v>
@@ -9141,7 +9265,7 @@
         <v>40.11494958459248</v>
       </c>
       <c r="J47">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K47" t="s">
         <v>161</v>
@@ -9211,7 +9335,7 @@
         <v>33.9729473260635</v>
       </c>
       <c r="J49">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K49" t="s">
         <v>162</v>
@@ -9246,7 +9370,7 @@
         <v>37.02109183728933</v>
       </c>
       <c r="J50">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K50" t="s">
         <v>162</v>
@@ -9281,7 +9405,7 @@
         <v>44.54939598291897</v>
       </c>
       <c r="J51">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K51" t="s">
         <v>161</v>
@@ -9316,7 +9440,7 @@
         <v>41.9093713425007</v>
       </c>
       <c r="J52">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K52" t="s">
         <v>161</v>
@@ -9351,7 +9475,7 @@
         <v>45.24736162443781</v>
       </c>
       <c r="J53">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K53" t="s">
         <v>161</v>
@@ -9386,7 +9510,7 @@
         <v>45.78635887349753</v>
       </c>
       <c r="J54">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K54" t="s">
         <v>161</v>
@@ -9421,7 +9545,7 @@
         <v>52.4694725609674</v>
       </c>
       <c r="J55">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K55" t="s">
         <v>161</v>
@@ -9456,7 +9580,7 @@
         <v>49.34571546247042</v>
       </c>
       <c r="J56">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K56" t="s">
         <v>161</v>
@@ -9491,7 +9615,7 @@
         <v>48.56229749649761</v>
       </c>
       <c r="J57">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K57" t="s">
         <v>161</v>
@@ -9508,7 +9632,7 @@
         <v>50.13999938964844</v>
       </c>
       <c r="D58">
-        <v>0.372</v>
+        <v>0.3721</v>
       </c>
       <c r="E58">
         <v>49.06369972229004</v>
@@ -9526,7 +9650,7 @@
         <v>50.89285279849747</v>
       </c>
       <c r="J58">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K58" t="s">
         <v>161</v>
@@ -9561,7 +9685,7 @@
         <v>51.77304029140512</v>
       </c>
       <c r="J59">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K59" t="s">
         <v>161</v>
@@ -9596,7 +9720,7 @@
         <v>55.20473843066302</v>
       </c>
       <c r="J60">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K60" t="s">
         <v>161</v>
@@ -9631,7 +9755,7 @@
         <v>59.28286837585451</v>
       </c>
       <c r="J61">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K61" t="s">
         <v>161</v>
@@ -9666,7 +9790,7 @@
         <v>57.49129481397203</v>
       </c>
       <c r="J62">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K62" t="s">
         <v>161</v>
@@ -9701,7 +9825,7 @@
         <v>60.49079921150475</v>
       </c>
       <c r="J63">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K63" t="s">
         <v>161</v>
@@ -9736,7 +9860,7 @@
         <v>63.52941319169427</v>
       </c>
       <c r="J64">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K64" t="s">
         <v>161</v>
@@ -9771,7 +9895,7 @@
         <v>61.87049520601642</v>
       </c>
       <c r="J65">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K65" t="s">
         <v>161</v>
@@ -9806,7 +9930,7 @@
         <v>58.27090592171268</v>
       </c>
       <c r="J66">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K66" t="s">
         <v>161</v>
@@ -9841,7 +9965,7 @@
         <v>61.54747452974244</v>
       </c>
       <c r="J67">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K67" t="s">
         <v>161</v>
@@ -9876,7 +10000,7 @@
         <v>69.46505928053598</v>
       </c>
       <c r="J68">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K68" t="s">
         <v>161</v>
@@ -9893,7 +10017,7 @@
         <v>8.024999618530273</v>
       </c>
       <c r="D69">
-        <v>0.3527</v>
+        <v>0.3528</v>
       </c>
       <c r="E69">
         <v>6.22210000038147</v>
@@ -9911,7 +10035,7 @@
         <v>62.92237220217377</v>
       </c>
       <c r="J69">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K69" t="s">
         <v>161</v>
@@ -9946,7 +10070,7 @@
         <v>67.58864039885938</v>
       </c>
       <c r="J70">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K70" t="s">
         <v>161</v>
@@ -9963,7 +10087,7 @@
         <v>78.55000305175781</v>
       </c>
       <c r="D71">
-        <v>0.3495</v>
+        <v>0.3496</v>
       </c>
       <c r="E71">
         <v>62.95691932678223</v>
@@ -9981,7 +10105,7 @@
         <v>65.88147838728383</v>
       </c>
       <c r="J71">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K71" t="s">
         <v>161</v>
@@ -10016,7 +10140,7 @@
         <v>58.07715318316384</v>
       </c>
       <c r="J72">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K72" t="s">
         <v>161</v>
@@ -10051,7 +10175,7 @@
         <v>69.011043961692</v>
       </c>
       <c r="J73">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K73" t="s">
         <v>161</v>
@@ -10086,7 +10210,7 @@
         <v>68.86465938081456</v>
       </c>
       <c r="J74">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K74" t="s">
         <v>161</v>
@@ -10103,7 +10227,7 @@
         <v>68.98000335693359</v>
       </c>
       <c r="D75">
-        <v>0.3407</v>
+        <v>0.3408</v>
       </c>
       <c r="E75">
         <v>43.68120010375976</v>
@@ -10121,7 +10245,7 @@
         <v>72.73146105094992</v>
       </c>
       <c r="J75">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K75" t="s">
         <v>161</v>
@@ -10156,7 +10280,7 @@
         <v>73.36374709939457</v>
       </c>
       <c r="J76">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K76" t="s">
         <v>161</v>
@@ -10191,7 +10315,7 @@
         <v>76.23765512710006</v>
       </c>
       <c r="J77">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K77" t="s">
         <v>161</v>
@@ -10226,7 +10350,7 @@
         <v>78.60111662018215</v>
       </c>
       <c r="J78">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K78" t="s">
         <v>161</v>
@@ -10261,7 +10385,7 @@
         <v>82.27680786422185</v>
       </c>
       <c r="J79">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K79" t="s">
         <v>161</v>
@@ -10296,7 +10420,7 @@
         <v>92.49556488986379</v>
       </c>
       <c r="J80">
-        <v>0.6603</v>
+        <v>0.6605</v>
       </c>
       <c r="K80" t="s">
         <v>161</v>
@@ -10361,22 +10485,22 @@
         <v>0.8158</v>
       </c>
       <c r="D2">
-        <v>0.2573</v>
+        <v>0.2566</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>7.27</v>
+        <v>7.28</v>
       </c>
       <c r="G2">
-        <v>584.4400000000001</v>
+        <v>587.8200000000001</v>
       </c>
       <c r="H2">
         <v>217.2599945068359</v>
       </c>
       <c r="I2">
-        <v>2.69</v>
+        <v>2.71</v>
       </c>
       <c r="J2" t="s">
         <v>153</v>
@@ -10399,16 +10523,16 @@
         <v>0.8028</v>
       </c>
       <c r="D3">
-        <v>0.4743</v>
+        <v>0.4729</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>5.06</v>
+        <v>5.08</v>
       </c>
       <c r="G3">
-        <v>406.78</v>
+        <v>410.18</v>
       </c>
       <c r="H3">
         <v>504.6749877929688</v>
@@ -10437,7 +10561,7 @@
         <v>0.6987</v>
       </c>
       <c r="D4">
-        <v>0.1222</v>
+        <v>0.1219</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -10446,13 +10570,13 @@
         <v>3.41</v>
       </c>
       <c r="G4">
-        <v>274.13</v>
+        <v>275.34</v>
       </c>
       <c r="H4">
         <v>79.44499969482422</v>
       </c>
       <c r="I4">
-        <v>3.45</v>
+        <v>3.47</v>
       </c>
       <c r="J4" t="s">
         <v>153</v>
@@ -10475,22 +10599,22 @@
         <v>0.8250999999999999</v>
       </c>
       <c r="D5">
-        <v>0.6728</v>
+        <v>0.6709000000000001</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3.24</v>
+        <v>3.26</v>
       </c>
       <c r="G5">
-        <v>260.47</v>
+        <v>263.23</v>
       </c>
       <c r="H5">
         <v>105.504997253418</v>
       </c>
       <c r="I5">
-        <v>2.47</v>
+        <v>2.49</v>
       </c>
       <c r="J5" t="s">
         <v>153</v>
@@ -10513,7 +10637,7 @@
         <v>0.6322</v>
       </c>
       <c r="D6">
-        <v>0.1066</v>
+        <v>0.1063</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -10522,13 +10646,13 @@
         <v>3.14</v>
       </c>
       <c r="G6">
-        <v>252.43</v>
+        <v>253.54</v>
       </c>
       <c r="H6">
         <v>756.3519897460938</v>
       </c>
       <c r="I6">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="J6" t="s">
         <v>153</v>
@@ -10548,10 +10672,10 @@
         <v>18</v>
       </c>
       <c r="C7">
-        <v>0.6524</v>
+        <v>0.6525</v>
       </c>
       <c r="D7">
-        <v>0.1517</v>
+        <v>0.1515</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -10560,13 +10684,13 @@
         <v>3.07</v>
       </c>
       <c r="G7">
-        <v>246.8</v>
+        <v>247.89</v>
       </c>
       <c r="H7">
         <v>289.6799926757812</v>
       </c>
       <c r="I7">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="J7" t="s">
         <v>153</v>
@@ -10589,7 +10713,7 @@
         <v>0.6333</v>
       </c>
       <c r="D8">
-        <v>0.1443</v>
+        <v>0.1439</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -10598,7 +10722,7 @@
         <v>3</v>
       </c>
       <c r="G8">
-        <v>241.17</v>
+        <v>242.24</v>
       </c>
       <c r="H8">
         <v>737.3900146484375</v>
@@ -10636,7 +10760,7 @@
         <v>2.92</v>
       </c>
       <c r="G9">
-        <v>234.74</v>
+        <v>235.78</v>
       </c>
       <c r="H9">
         <v>378.1099853515625</v>
@@ -10665,7 +10789,7 @@
         <v>0.6245000000000001</v>
       </c>
       <c r="D10">
-        <v>0.1759</v>
+        <v>0.1764</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -10674,7 +10798,7 @@
         <v>2.85</v>
       </c>
       <c r="G10">
-        <v>229.11</v>
+        <v>230.12</v>
       </c>
       <c r="H10">
         <v>311.3699951171875</v>
@@ -10703,7 +10827,7 @@
         <v>0.6708</v>
       </c>
       <c r="D11">
-        <v>0.2467</v>
+        <v>0.2484</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -10712,7 +10836,7 @@
         <v>2.8</v>
       </c>
       <c r="G11">
-        <v>225.09</v>
+        <v>226.09</v>
       </c>
       <c r="H11">
         <v>400.5350036621094</v>
@@ -10741,16 +10865,16 @@
         <v>0.6714</v>
       </c>
       <c r="D12">
-        <v>0.2589</v>
+        <v>0.2586</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12">
-        <v>2.76</v>
+        <v>2.77</v>
       </c>
       <c r="G12">
-        <v>221.88</v>
+        <v>223.66</v>
       </c>
       <c r="H12">
         <v>452.6400146484375</v>
@@ -10776,19 +10900,19 @@
         <v>18</v>
       </c>
       <c r="C13">
-        <v>0.6448</v>
+        <v>0.6449</v>
       </c>
       <c r="D13">
-        <v>0.2471</v>
+        <v>0.2476</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
       <c r="F13">
-        <v>2.7</v>
+        <v>2.69</v>
       </c>
       <c r="G13">
-        <v>217.06</v>
+        <v>217.2</v>
       </c>
       <c r="H13">
         <v>599.510009765625</v>
@@ -10808,31 +10932,31 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="B14" t="s">
         <v>18</v>
       </c>
       <c r="C14">
-        <v>0.6313</v>
+        <v>0.6625</v>
       </c>
       <c r="D14">
-        <v>0.2495</v>
+        <v>0.2822</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
       <c r="F14">
-        <v>2.63</v>
+        <v>2.64</v>
       </c>
       <c r="G14">
-        <v>211.43</v>
+        <v>213.17</v>
       </c>
       <c r="H14">
-        <v>120.9800033569336</v>
+        <v>418.6000061035156</v>
       </c>
       <c r="I14">
-        <v>1.75</v>
+        <v>0.51</v>
       </c>
       <c r="J14" t="s">
         <v>153</v>
@@ -10846,31 +10970,31 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="B15" t="s">
         <v>18</v>
       </c>
       <c r="C15">
-        <v>0.6625</v>
+        <v>0.6313</v>
       </c>
       <c r="D15">
-        <v>0.2827</v>
+        <v>0.2518</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
       <c r="F15">
-        <v>2.63</v>
+        <v>2.62</v>
       </c>
       <c r="G15">
-        <v>211.43</v>
+        <v>211.55</v>
       </c>
       <c r="H15">
-        <v>418.6000061035156</v>
+        <v>120.9800033569336</v>
       </c>
       <c r="I15">
-        <v>0.51</v>
+        <v>1.75</v>
       </c>
       <c r="J15" t="s">
         <v>153</v>
@@ -10893,7 +11017,7 @@
         <v>0.6421</v>
       </c>
       <c r="D16">
-        <v>0.2724</v>
+        <v>0.2738</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -10902,7 +11026,7 @@
         <v>2.59</v>
       </c>
       <c r="G16">
-        <v>208.21</v>
+        <v>209.13</v>
       </c>
       <c r="H16">
         <v>566.0499877929688</v>
@@ -10931,7 +11055,7 @@
         <v>0.6666</v>
       </c>
       <c r="D17">
-        <v>0.3203</v>
+        <v>0.3213</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -10940,13 +11064,13 @@
         <v>2.51</v>
       </c>
       <c r="G17">
-        <v>201.78</v>
+        <v>202.67</v>
       </c>
       <c r="H17">
         <v>1616.579956054688</v>
       </c>
       <c r="I17">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="J17" t="s">
         <v>153</v>
@@ -10978,13 +11102,13 @@
         <v>2.44</v>
       </c>
       <c r="G18">
-        <v>196.15</v>
+        <v>197.02</v>
       </c>
       <c r="H18">
         <v>136.8999938964844</v>
       </c>
       <c r="I18">
-        <v>1.43</v>
+        <v>1.44</v>
       </c>
       <c r="J18" t="s">
         <v>153</v>
@@ -11004,19 +11128,19 @@
         <v>18</v>
       </c>
       <c r="C19">
-        <v>0.6627</v>
+        <v>0.6627999999999999</v>
       </c>
       <c r="D19">
-        <v>0.3569</v>
+        <v>0.3586</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
       <c r="F19">
-        <v>2.37</v>
+        <v>2.36</v>
       </c>
       <c r="G19">
-        <v>190.53</v>
+        <v>190.56</v>
       </c>
       <c r="H19">
         <v>437.3999938964844</v>
@@ -11042,10 +11166,10 @@
         <v>18</v>
       </c>
       <c r="C20">
-        <v>0.6621</v>
+        <v>0.6622</v>
       </c>
       <c r="D20">
-        <v>0.3757</v>
+        <v>0.3761</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -11054,7 +11178,7 @@
         <v>2.29</v>
       </c>
       <c r="G20">
-        <v>184.1</v>
+        <v>184.91</v>
       </c>
       <c r="H20">
         <v>1930.010009765625</v>
@@ -11080,10 +11204,10 @@
         <v>18</v>
       </c>
       <c r="C21">
-        <v>0.6253</v>
+        <v>0.6254</v>
       </c>
       <c r="D21">
-        <v>0.3667</v>
+        <v>0.3672</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -11092,13 +11216,13 @@
         <v>2.2</v>
       </c>
       <c r="G21">
-        <v>176.86</v>
+        <v>177.64</v>
       </c>
       <c r="H21">
         <v>279.1600036621094</v>
       </c>
       <c r="I21">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="J21" t="s">
         <v>153</v>
@@ -11118,10 +11242,10 @@
         <v>18</v>
       </c>
       <c r="C22">
-        <v>0.649</v>
+        <v>0.6491</v>
       </c>
       <c r="D22">
-        <v>0.3975</v>
+        <v>0.3971</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -11130,7 +11254,7 @@
         <v>2.17</v>
       </c>
       <c r="G22">
-        <v>174.45</v>
+        <v>175.22</v>
       </c>
       <c r="H22">
         <v>160.1600036621094</v>
@@ -11159,7 +11283,7 @@
         <v>0.6884</v>
       </c>
       <c r="D23">
-        <v>0.4345</v>
+        <v>0.4344</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -11168,13 +11292,13 @@
         <v>2.16</v>
       </c>
       <c r="G23">
-        <v>173.64</v>
+        <v>174.41</v>
       </c>
       <c r="H23">
         <v>313.2200012207031</v>
       </c>
       <c r="I23">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="J23" t="s">
         <v>153</v>
@@ -11197,22 +11321,22 @@
         <v>0.6871</v>
       </c>
       <c r="D24">
-        <v>0.4402</v>
+        <v>0.4392</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
       <c r="F24">
-        <v>2.13</v>
+        <v>2.14</v>
       </c>
       <c r="G24">
-        <v>171.23</v>
+        <v>172.79</v>
       </c>
       <c r="H24">
         <v>192.1600036621094</v>
       </c>
       <c r="I24">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="J24" t="s">
         <v>153</v>
@@ -11226,31 +11350,31 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="B25" t="s">
         <v>18</v>
       </c>
       <c r="C25">
-        <v>0.6445</v>
+        <v>0.6128</v>
       </c>
       <c r="D25">
-        <v>0.4439</v>
+        <v>0.4227</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
       <c r="F25">
-        <v>1.99</v>
+        <v>1.96</v>
       </c>
       <c r="G25">
-        <v>159.98</v>
+        <v>158.26</v>
       </c>
       <c r="H25">
-        <v>204.1499938964844</v>
+        <v>726.155029296875</v>
       </c>
       <c r="I25">
-        <v>0.78</v>
+        <v>0.22</v>
       </c>
       <c r="J25" t="s">
         <v>153</v>
@@ -11264,31 +11388,31 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="B26" t="s">
         <v>18</v>
       </c>
       <c r="C26">
-        <v>0.6127</v>
+        <v>0.6435999999999999</v>
       </c>
       <c r="D26">
-        <v>0.4215</v>
+        <v>0.4764</v>
       </c>
       <c r="E26">
         <v>0</v>
       </c>
       <c r="F26">
-        <v>1.97</v>
+        <v>1.87</v>
       </c>
       <c r="G26">
-        <v>158.37</v>
+        <v>150.99</v>
       </c>
       <c r="H26">
-        <v>726.155029296875</v>
+        <v>38.50500106811523</v>
       </c>
       <c r="I26">
-        <v>0.22</v>
+        <v>3.92</v>
       </c>
       <c r="J26" t="s">
         <v>153</v>
@@ -11302,31 +11426,31 @@
     </row>
     <row r="27" spans="1:12">
       <c r="A27" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B27" t="s">
         <v>18</v>
       </c>
       <c r="C27">
-        <v>0.6435999999999999</v>
+        <v>0.6445</v>
       </c>
       <c r="D27">
-        <v>0.4773</v>
+        <v>0.4971</v>
       </c>
       <c r="E27">
         <v>0</v>
       </c>
       <c r="F27">
-        <v>1.87</v>
+        <v>1.8</v>
       </c>
       <c r="G27">
-        <v>150.33</v>
+        <v>145.34</v>
       </c>
       <c r="H27">
-        <v>38.50500106811523</v>
+        <v>204.1499938964844</v>
       </c>
       <c r="I27">
-        <v>3.9</v>
+        <v>0.71</v>
       </c>
       <c r="J27" t="s">
         <v>153</v>
@@ -11349,22 +11473,22 @@
         <v>0.6895</v>
       </c>
       <c r="D28">
-        <v>0.5324</v>
+        <v>0.5309</v>
       </c>
       <c r="E28">
         <v>0</v>
       </c>
       <c r="F28">
-        <v>1.79</v>
+        <v>1.8</v>
       </c>
       <c r="G28">
-        <v>143.9</v>
+        <v>145.34</v>
       </c>
       <c r="H28">
         <v>118.0699996948242</v>
       </c>
       <c r="I28">
-        <v>1.22</v>
+        <v>1.23</v>
       </c>
       <c r="J28" t="s">
         <v>153</v>
@@ -11387,7 +11511,7 @@
         <v>0.6356000000000001</v>
       </c>
       <c r="D29">
-        <v>0.5026</v>
+        <v>0.5011</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -11396,13 +11520,13 @@
         <v>1.76</v>
       </c>
       <c r="G29">
-        <v>141.49</v>
+        <v>142.11</v>
       </c>
       <c r="H29">
         <v>238.2949981689453</v>
       </c>
       <c r="I29">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="J29" t="s">
         <v>153</v>
@@ -11422,10 +11546,10 @@
         <v>18</v>
       </c>
       <c r="C30">
-        <v>0.6236</v>
+        <v>0.6237</v>
       </c>
       <c r="D30">
-        <v>0.5076000000000001</v>
+        <v>0.5078</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -11434,7 +11558,7 @@
         <v>1.7</v>
       </c>
       <c r="G30">
-        <v>136.66</v>
+        <v>137.27</v>
       </c>
       <c r="H30">
         <v>416.2999877929688</v>
@@ -11463,7 +11587,7 @@
         <v>0.6249</v>
       </c>
       <c r="D31">
-        <v>0.5285</v>
+        <v>0.5269</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -11472,7 +11596,7 @@
         <v>1.64</v>
       </c>
       <c r="G31">
-        <v>131.84</v>
+        <v>132.42</v>
       </c>
       <c r="H31">
         <v>351.0299987792969</v>
@@ -11501,7 +11625,7 @@
         <v>0.6441</v>
       </c>
       <c r="D32">
-        <v>0.5443</v>
+        <v>0.5427999999999999</v>
       </c>
       <c r="E32">
         <v>0</v>
@@ -11510,7 +11634,7 @@
         <v>1.63</v>
       </c>
       <c r="G32">
-        <v>131.04</v>
+        <v>131.61</v>
       </c>
       <c r="H32">
         <v>946.5999755859375</v>
@@ -11539,7 +11663,7 @@
         <v>0.627</v>
       </c>
       <c r="D33">
-        <v>0.5462</v>
+        <v>0.5458</v>
       </c>
       <c r="E33">
         <v>0</v>
@@ -11548,7 +11672,7 @@
         <v>1.58</v>
       </c>
       <c r="G33">
-        <v>127.02</v>
+        <v>127.58</v>
       </c>
       <c r="H33">
         <v>243.2799987792969</v>
@@ -11577,16 +11701,16 @@
         <v>0.4589</v>
       </c>
       <c r="D34">
-        <v>0.3435</v>
+        <v>0.343</v>
       </c>
       <c r="E34">
         <v>0</v>
       </c>
       <c r="F34">
-        <v>1.44</v>
+        <v>1.45</v>
       </c>
       <c r="G34">
-        <v>115.76</v>
+        <v>117.08</v>
       </c>
       <c r="H34">
         <v>434.2398986816406</v>
@@ -11615,7 +11739,7 @@
         <v>0.6681</v>
       </c>
       <c r="D35">
-        <v>0.6424</v>
+        <v>0.641</v>
       </c>
       <c r="E35">
         <v>0</v>
@@ -11624,13 +11748,13 @@
         <v>1.33</v>
       </c>
       <c r="G35">
-        <v>106.92</v>
+        <v>107.39</v>
       </c>
       <c r="H35">
         <v>1646.010009765625</v>
       </c>
       <c r="I35">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="J35" t="s">
         <v>153</v>
@@ -11653,7 +11777,7 @@
         <v>0.4093</v>
       </c>
       <c r="D36">
-        <v>0.3324</v>
+        <v>0.3318</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -11662,7 +11786,7 @@
         <v>1.31</v>
       </c>
       <c r="G36">
-        <v>105.31</v>
+        <v>105.78</v>
       </c>
       <c r="H36">
         <v>627.8200073242188</v>
@@ -11688,25 +11812,25 @@
         <v>18</v>
       </c>
       <c r="C37">
-        <v>0.6529</v>
+        <v>0.6533</v>
       </c>
       <c r="D37">
-        <v>0.2408</v>
+        <v>0.2402</v>
       </c>
       <c r="E37">
-        <v>0.4285</v>
+        <v>0.4272</v>
       </c>
       <c r="F37">
-        <v>1.22</v>
+        <v>1.23</v>
       </c>
       <c r="G37">
-        <v>98.08</v>
+        <v>99.31999999999999</v>
       </c>
       <c r="H37">
         <v>270.2804870605469</v>
       </c>
       <c r="I37">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="J37" t="s">
         <v>153</v>
@@ -11729,22 +11853,22 @@
         <v>0.7183</v>
       </c>
       <c r="D38">
-        <v>0.7488</v>
+        <v>0.7475000000000001</v>
       </c>
       <c r="E38">
         <v>0</v>
       </c>
       <c r="F38">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="G38">
-        <v>80.39</v>
+        <v>81.55</v>
       </c>
       <c r="H38">
         <v>32.22999954223633</v>
       </c>
       <c r="I38">
-        <v>2.49</v>
+        <v>2.53</v>
       </c>
       <c r="J38" t="s">
         <v>153</v>
@@ -11764,10 +11888,10 @@
         <v>18</v>
       </c>
       <c r="C39">
-        <v>0.6509</v>
+        <v>0.651</v>
       </c>
       <c r="D39">
-        <v>0.7318</v>
+        <v>0.7301</v>
       </c>
       <c r="E39">
         <v>0</v>
@@ -11776,7 +11900,7 @@
         <v>0.97</v>
       </c>
       <c r="G39">
-        <v>77.98</v>
+        <v>78.31999999999999</v>
       </c>
       <c r="H39">
         <v>229.1600036621094</v>
@@ -11805,7 +11929,7 @@
         <v>0.6251</v>
       </c>
       <c r="D40">
-        <v>0.7252</v>
+        <v>0.7268</v>
       </c>
       <c r="E40">
         <v>0</v>
@@ -11814,7 +11938,7 @@
         <v>0.95</v>
       </c>
       <c r="G40">
-        <v>76.37</v>
+        <v>76.70999999999999</v>
       </c>
       <c r="H40">
         <v>335.5</v>
@@ -11843,16 +11967,16 @@
         <v>0.4099</v>
       </c>
       <c r="D41">
-        <v>0.317</v>
+        <v>0.32</v>
       </c>
       <c r="E41">
         <v>0</v>
       </c>
       <c r="F41">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="G41">
-        <v>71.55</v>
+        <v>71.06</v>
       </c>
       <c r="H41">
         <v>842.4000244140625</v>
@@ -11881,7 +12005,7 @@
         <v>0.6493</v>
       </c>
       <c r="D42">
-        <v>0.7651</v>
+        <v>0.7637</v>
       </c>
       <c r="E42">
         <v>0</v>
@@ -11890,13 +12014,13 @@
         <v>0.85</v>
       </c>
       <c r="G42">
-        <v>68.33</v>
+        <v>68.63</v>
       </c>
       <c r="H42">
         <v>17.04999923706055</v>
       </c>
       <c r="I42">
-        <v>4.01</v>
+        <v>4.03</v>
       </c>
       <c r="J42" t="s">
         <v>153</v>
@@ -11910,31 +12034,31 @@
     </row>
     <row r="43" spans="1:12">
       <c r="A43" t="s">
-        <v>71</v>
+        <v>110</v>
       </c>
       <c r="B43" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="C43">
-        <v>0.8011</v>
+        <v>0.4012</v>
       </c>
       <c r="D43">
-        <v>0.8985</v>
+        <v>0.3581</v>
       </c>
       <c r="E43">
         <v>0</v>
       </c>
       <c r="F43">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="G43">
-        <v>65.12</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="H43">
-        <v>10.6201000213623</v>
+        <v>477.3900146484375</v>
       </c>
       <c r="I43">
-        <v>6.13</v>
+        <v>0.14</v>
       </c>
       <c r="J43" t="s">
         <v>153</v>
@@ -11943,36 +12067,36 @@
         <v>1.2</v>
       </c>
       <c r="L43" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="44" spans="1:12">
       <c r="A44" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B44" t="s">
         <v>143</v>
       </c>
       <c r="C44">
-        <v>0.4012</v>
+        <v>0.4315</v>
       </c>
       <c r="D44">
-        <v>0.3589</v>
+        <v>0.6191</v>
       </c>
       <c r="E44">
         <v>0</v>
       </c>
       <c r="F44">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="G44">
-        <v>65.12</v>
+        <v>63.79</v>
       </c>
       <c r="H44">
-        <v>477.3900146484375</v>
+        <v>92.66010284423828</v>
       </c>
       <c r="I44">
-        <v>0.14</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="J44" t="s">
         <v>153</v>
@@ -11981,7 +12105,7 @@
         <v>1.2</v>
       </c>
       <c r="L44" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -11995,22 +12119,22 @@
         <v>0.6788999999999999</v>
       </c>
       <c r="D45">
-        <v>0.7842</v>
+        <v>0.7948</v>
       </c>
       <c r="E45">
         <v>0</v>
       </c>
       <c r="F45">
-        <v>0.8100000000000001</v>
+        <v>0.77</v>
       </c>
       <c r="G45">
-        <v>65.12</v>
+        <v>62.17</v>
       </c>
       <c r="H45">
         <v>92</v>
       </c>
       <c r="I45">
-        <v>0.71</v>
+        <v>0.68</v>
       </c>
       <c r="J45" t="s">
         <v>153</v>
@@ -12024,31 +12148,31 @@
     </row>
     <row r="46" spans="1:12">
       <c r="A46" t="s">
-        <v>108</v>
+        <v>71</v>
       </c>
       <c r="B46" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="C46">
-        <v>0.4315</v>
+        <v>0.8007</v>
       </c>
       <c r="D46">
-        <v>0.6197</v>
+        <v>0.9114</v>
       </c>
       <c r="E46">
         <v>0</v>
       </c>
       <c r="F46">
-        <v>0.79</v>
+        <v>0.7</v>
       </c>
       <c r="G46">
-        <v>63.51</v>
+        <v>56.52</v>
       </c>
       <c r="H46">
-        <v>92.66010284423828</v>
+        <v>10.6201000213623</v>
       </c>
       <c r="I46">
-        <v>0.6899999999999999</v>
+        <v>5.32</v>
       </c>
       <c r="J46" t="s">
         <v>153</v>
@@ -12057,7 +12181,7 @@
         <v>1.2</v>
       </c>
       <c r="L46" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -12071,7 +12195,7 @@
         <v>0.385</v>
       </c>
       <c r="D47">
-        <v>0.2378</v>
+        <v>0.2386</v>
       </c>
       <c r="E47">
         <v>0</v>
@@ -12080,7 +12204,7 @@
         <v>0.24</v>
       </c>
       <c r="G47">
-        <v>19.29</v>
+        <v>19.38</v>
       </c>
       <c r="H47">
         <v>86.90000152587891</v>
@@ -12109,7 +12233,7 @@
         <v>0.3491</v>
       </c>
       <c r="D48">
-        <v>0.2971</v>
+        <v>0.2967</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -12118,7 +12242,7 @@
         <v>0.2</v>
       </c>
       <c r="G48">
-        <v>16.08</v>
+        <v>16.15</v>
       </c>
       <c r="H48">
         <v>81.58999633789062</v>
@@ -12147,7 +12271,7 @@
         <v>0.3449</v>
       </c>
       <c r="D49">
-        <v>0.2911</v>
+        <v>0.2928</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -12156,7 +12280,7 @@
         <v>0.19</v>
       </c>
       <c r="G49">
-        <v>15.27</v>
+        <v>15.34</v>
       </c>
       <c r="H49">
         <v>442.6698913574219</v>
@@ -12194,7 +12318,7 @@
         <v>0.19</v>
       </c>
       <c r="G50">
-        <v>15.27</v>
+        <v>15.34</v>
       </c>
       <c r="H50">
         <v>376.1700134277344</v>
@@ -12214,31 +12338,31 @@
     </row>
     <row r="51" spans="1:12">
       <c r="A51" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B51" t="s">
         <v>144</v>
       </c>
       <c r="C51">
-        <v>0.3778</v>
+        <v>0.3765</v>
       </c>
       <c r="D51">
-        <v>0.3827</v>
+        <v>0.4146</v>
       </c>
       <c r="E51">
         <v>0</v>
       </c>
       <c r="F51">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="G51">
-        <v>15.27</v>
+        <v>14.53</v>
       </c>
       <c r="H51">
-        <v>256.6799926757812</v>
+        <v>16.40999984741211</v>
       </c>
       <c r="I51">
-        <v>0.06</v>
+        <v>0.89</v>
       </c>
       <c r="J51" t="s">
         <v>153</v>
@@ -12252,16 +12376,16 @@
     </row>
     <row r="52" spans="1:12">
       <c r="A52" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B52" t="s">
         <v>144</v>
       </c>
       <c r="C52">
-        <v>0.3765</v>
+        <v>0.3496</v>
       </c>
       <c r="D52">
-        <v>0.4138</v>
+        <v>0.359</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -12270,13 +12394,13 @@
         <v>0.18</v>
       </c>
       <c r="G52">
-        <v>14.47</v>
+        <v>14.53</v>
       </c>
       <c r="H52">
-        <v>16.40999984741211</v>
+        <v>78.55000305175781</v>
       </c>
       <c r="I52">
-        <v>0.88</v>
+        <v>0.18</v>
       </c>
       <c r="J52" t="s">
         <v>153</v>
@@ -12290,16 +12414,16 @@
     </row>
     <row r="53" spans="1:12">
       <c r="A53" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="B53" t="s">
         <v>144</v>
       </c>
       <c r="C53">
-        <v>0.3495</v>
+        <v>0.369</v>
       </c>
       <c r="D53">
-        <v>0.3559</v>
+        <v>0.3835</v>
       </c>
       <c r="E53">
         <v>0</v>
@@ -12308,13 +12432,13 @@
         <v>0.18</v>
       </c>
       <c r="G53">
-        <v>14.47</v>
+        <v>14.53</v>
       </c>
       <c r="H53">
-        <v>78.55000305175781</v>
+        <v>42.81000137329102</v>
       </c>
       <c r="I53">
-        <v>0.18</v>
+        <v>0.34</v>
       </c>
       <c r="J53" t="s">
         <v>153</v>
@@ -12328,16 +12452,16 @@
     </row>
     <row r="54" spans="1:12">
       <c r="A54" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B54" t="s">
         <v>144</v>
       </c>
       <c r="C54">
-        <v>0.369</v>
+        <v>0.3778</v>
       </c>
       <c r="D54">
-        <v>0.3842</v>
+        <v>0.3851</v>
       </c>
       <c r="E54">
         <v>0</v>
@@ -12346,13 +12470,13 @@
         <v>0.18</v>
       </c>
       <c r="G54">
-        <v>14.47</v>
+        <v>14.53</v>
       </c>
       <c r="H54">
-        <v>42.81000137329102</v>
+        <v>256.6799926757812</v>
       </c>
       <c r="I54">
-        <v>0.34</v>
+        <v>0.06</v>
       </c>
       <c r="J54" t="s">
         <v>153</v>
@@ -12375,7 +12499,7 @@
         <v>0.3863</v>
       </c>
       <c r="D55">
-        <v>0.4354</v>
+        <v>0.435</v>
       </c>
       <c r="E55">
         <v>0</v>
@@ -12384,7 +12508,7 @@
         <v>0.18</v>
       </c>
       <c r="G55">
-        <v>14.47</v>
+        <v>14.53</v>
       </c>
       <c r="H55">
         <v>286.9700012207031</v>
@@ -12413,7 +12537,7 @@
         <v>0.3325</v>
       </c>
       <c r="D56">
-        <v>0.3907</v>
+        <v>0.3899</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -12422,7 +12546,7 @@
         <v>0.16</v>
       </c>
       <c r="G56">
-        <v>12.86</v>
+        <v>12.92</v>
       </c>
       <c r="H56">
         <v>297.8349914550781</v>
@@ -12451,7 +12575,7 @@
         <v>0.3971</v>
       </c>
       <c r="D57">
-        <v>0.5256999999999999</v>
+        <v>0.5245</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -12460,7 +12584,7 @@
         <v>0.15</v>
       </c>
       <c r="G57">
-        <v>12.06</v>
+        <v>12.11</v>
       </c>
       <c r="H57">
         <v>46.2599983215332</v>
@@ -12489,7 +12613,7 @@
         <v>0.3798</v>
       </c>
       <c r="D58">
-        <v>0.5144</v>
+        <v>0.5154</v>
       </c>
       <c r="E58">
         <v>0</v>
@@ -12498,7 +12622,7 @@
         <v>0.15</v>
       </c>
       <c r="G58">
-        <v>12.06</v>
+        <v>12.11</v>
       </c>
       <c r="H58">
         <v>71.58999633789062</v>
@@ -12527,7 +12651,7 @@
         <v>0.3554</v>
       </c>
       <c r="D59">
-        <v>0.5096000000000001</v>
+        <v>0.5101</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -12536,7 +12660,7 @@
         <v>0.14</v>
       </c>
       <c r="G59">
-        <v>11.25</v>
+        <v>11.3</v>
       </c>
       <c r="H59">
         <v>109.3625030517578</v>
@@ -12565,7 +12689,7 @@
         <v>0.3507</v>
       </c>
       <c r="D60">
-        <v>0.4861</v>
+        <v>0.4859</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -12574,7 +12698,7 @@
         <v>0.14</v>
       </c>
       <c r="G60">
-        <v>11.25</v>
+        <v>11.3</v>
       </c>
       <c r="H60">
         <v>223.4850006103516</v>
@@ -12603,7 +12727,7 @@
         <v>0.3615</v>
       </c>
       <c r="D61">
-        <v>0.5157</v>
+        <v>0.5199</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -12612,7 +12736,7 @@
         <v>0.14</v>
       </c>
       <c r="G61">
-        <v>11.25</v>
+        <v>11.3</v>
       </c>
       <c r="H61">
         <v>144.8500061035156</v>
@@ -12638,10 +12762,10 @@
         <v>144</v>
       </c>
       <c r="C62">
-        <v>0.372</v>
+        <v>0.3721</v>
       </c>
       <c r="D62">
-        <v>0.5313</v>
+        <v>0.5316</v>
       </c>
       <c r="E62">
         <v>0</v>
@@ -12650,13 +12774,13 @@
         <v>0.14</v>
       </c>
       <c r="G62">
-        <v>11.25</v>
+        <v>11.3</v>
       </c>
       <c r="H62">
         <v>50.13999938964844</v>
       </c>
       <c r="I62">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="J62" t="s">
         <v>153</v>
@@ -12679,7 +12803,7 @@
         <v>0.3629</v>
       </c>
       <c r="D63">
-        <v>0.5326</v>
+        <v>0.5329</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -12688,13 +12812,13 @@
         <v>0.14</v>
       </c>
       <c r="G63">
-        <v>11.25</v>
+        <v>11.3</v>
       </c>
       <c r="H63">
         <v>3.535000085830688</v>
       </c>
       <c r="I63">
-        <v>3.18</v>
+        <v>3.2</v>
       </c>
       <c r="J63" t="s">
         <v>153</v>
@@ -12717,7 +12841,7 @@
         <v>0.3571</v>
       </c>
       <c r="D64">
-        <v>0.5459000000000001</v>
+        <v>0.5464</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -12726,13 +12850,13 @@
         <v>0.13</v>
       </c>
       <c r="G64">
-        <v>10.45</v>
+        <v>10.5</v>
       </c>
       <c r="H64">
         <v>24.07999992370605</v>
       </c>
       <c r="I64">
-        <v>0.43</v>
+        <v>0.44</v>
       </c>
       <c r="J64" t="s">
         <v>153</v>
@@ -12755,7 +12879,7 @@
         <v>0.3647</v>
       </c>
       <c r="D65">
-        <v>0.6032999999999999</v>
+        <v>0.6021</v>
       </c>
       <c r="E65">
         <v>0</v>
@@ -12764,7 +12888,7 @@
         <v>0.12</v>
       </c>
       <c r="G65">
-        <v>9.65</v>
+        <v>9.69</v>
       </c>
       <c r="H65">
         <v>326.5499877929688</v>
@@ -12793,7 +12917,7 @@
         <v>0.3866</v>
       </c>
       <c r="D66">
-        <v>0.6338</v>
+        <v>0.6384</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -12802,7 +12926,7 @@
         <v>0.11</v>
       </c>
       <c r="G66">
-        <v>8.84</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="H66">
         <v>138.6849975585938</v>
@@ -12831,7 +12955,7 @@
         <v>0.3343</v>
       </c>
       <c r="D67">
-        <v>0.5817</v>
+        <v>0.5851</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -12840,7 +12964,7 @@
         <v>0.11</v>
       </c>
       <c r="G67">
-        <v>8.84</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="H67">
         <v>122.8566970825195</v>
@@ -12869,7 +12993,7 @@
         <v>0.3627</v>
       </c>
       <c r="D68">
-        <v>0.6091</v>
+        <v>0.6143999999999999</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -12878,7 +13002,7 @@
         <v>0.11</v>
       </c>
       <c r="G68">
-        <v>8.84</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="H68">
         <v>11.64500045776367</v>
@@ -12907,7 +13031,7 @@
         <v>0.3557</v>
       </c>
       <c r="D69">
-        <v>0.5955</v>
+        <v>0.5954</v>
       </c>
       <c r="E69">
         <v>0</v>
@@ -12916,13 +13040,13 @@
         <v>0.11</v>
       </c>
       <c r="G69">
-        <v>8.84</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="H69">
         <v>10.85499954223633</v>
       </c>
       <c r="I69">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="J69" t="s">
         <v>153</v>
@@ -12945,7 +13069,7 @@
         <v>0.3691</v>
       </c>
       <c r="D70">
-        <v>0.6439</v>
+        <v>0.6434</v>
       </c>
       <c r="E70">
         <v>0</v>
@@ -12954,7 +13078,7 @@
         <v>0.1</v>
       </c>
       <c r="G70">
-        <v>8.039999999999999</v>
+        <v>8.07</v>
       </c>
       <c r="H70">
         <v>8.979999542236328</v>
@@ -12980,10 +13104,10 @@
         <v>144</v>
       </c>
       <c r="C71">
-        <v>0.3527</v>
+        <v>0.3528</v>
       </c>
       <c r="D71">
-        <v>0.6412</v>
+        <v>0.6419</v>
       </c>
       <c r="E71">
         <v>0</v>
@@ -12992,13 +13116,13 @@
         <v>0.1</v>
       </c>
       <c r="G71">
-        <v>8.039999999999999</v>
+        <v>8.07</v>
       </c>
       <c r="H71">
         <v>8.024999618530273</v>
       </c>
       <c r="I71">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="J71" t="s">
         <v>153</v>
@@ -13021,7 +13145,7 @@
         <v>0.3364</v>
       </c>
       <c r="D72">
-        <v>0.6568000000000001</v>
+        <v>0.6555</v>
       </c>
       <c r="E72">
         <v>0</v>
@@ -13030,7 +13154,7 @@
         <v>0.09</v>
       </c>
       <c r="G72">
-        <v>7.24</v>
+        <v>7.27</v>
       </c>
       <c r="H72">
         <v>613.1300048828125</v>
@@ -13059,7 +13183,7 @@
         <v>0.34</v>
       </c>
       <c r="D73">
-        <v>0.6641</v>
+        <v>0.6649</v>
       </c>
       <c r="E73">
         <v>0</v>
@@ -13068,7 +13192,7 @@
         <v>0.09</v>
       </c>
       <c r="G73">
-        <v>7.24</v>
+        <v>7.27</v>
       </c>
       <c r="H73">
         <v>45.6150016784668</v>
@@ -13097,7 +13221,7 @@
         <v>0.348</v>
       </c>
       <c r="D74">
-        <v>0.6959</v>
+        <v>0.6954</v>
       </c>
       <c r="E74">
         <v>0</v>
@@ -13106,13 +13230,13 @@
         <v>0.09</v>
       </c>
       <c r="G74">
-        <v>7.24</v>
+        <v>7.27</v>
       </c>
       <c r="H74">
         <v>5.026599884033203</v>
       </c>
       <c r="I74">
-        <v>1.44</v>
+        <v>1.45</v>
       </c>
       <c r="J74" t="s">
         <v>153</v>
@@ -13135,7 +13259,7 @@
         <v>0.3132</v>
       </c>
       <c r="D75">
-        <v>0.6752</v>
+        <v>0.6778</v>
       </c>
       <c r="E75">
         <v>0</v>
@@ -13144,7 +13268,7 @@
         <v>0.08</v>
       </c>
       <c r="G75">
-        <v>6.43</v>
+        <v>6.46</v>
       </c>
       <c r="H75">
         <v>253.3600006103516</v>
@@ -13170,10 +13294,10 @@
         <v>144</v>
       </c>
       <c r="C76">
-        <v>0.3407</v>
+        <v>0.3408</v>
       </c>
       <c r="D76">
-        <v>0.7524999999999999</v>
+        <v>0.7504999999999999</v>
       </c>
       <c r="E76">
         <v>0</v>
@@ -13182,7 +13306,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="G76">
-        <v>5.63</v>
+        <v>5.65</v>
       </c>
       <c r="H76">
         <v>68.98000335693359</v>
@@ -13202,16 +13326,16 @@
     </row>
     <row r="77" spans="1:12">
       <c r="A77" t="s">
-        <v>117</v>
+        <v>78</v>
       </c>
       <c r="B77" t="s">
-        <v>144</v>
+        <v>18</v>
       </c>
       <c r="C77">
-        <v>0.3768</v>
+        <v>0.675</v>
       </c>
       <c r="D77">
-        <v>0.7939000000000001</v>
+        <v>0.9833</v>
       </c>
       <c r="E77">
         <v>0</v>
@@ -13220,13 +13344,13 @@
         <v>0.06</v>
       </c>
       <c r="G77">
-        <v>4.82</v>
+        <v>4.84</v>
       </c>
       <c r="H77">
-        <v>12.4601001739502</v>
+        <v>156.1300048828125</v>
       </c>
       <c r="I77">
-        <v>0.39</v>
+        <v>0.03</v>
       </c>
       <c r="J77" t="s">
         <v>153</v>
@@ -13235,36 +13359,36 @@
         <v>1.2</v>
       </c>
       <c r="L77" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="78" spans="1:12">
       <c r="A78" t="s">
-        <v>78</v>
+        <v>117</v>
       </c>
       <c r="B78" t="s">
-        <v>18</v>
+        <v>144</v>
       </c>
       <c r="C78">
-        <v>0.6749000000000001</v>
+        <v>0.3768</v>
       </c>
       <c r="D78">
-        <v>0.9859</v>
+        <v>0.7959000000000001</v>
       </c>
       <c r="E78">
         <v>0</v>
       </c>
       <c r="F78">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="G78">
-        <v>4.02</v>
+        <v>4.84</v>
       </c>
       <c r="H78">
-        <v>156.1300048828125</v>
+        <v>12.4601001739502</v>
       </c>
       <c r="I78">
-        <v>0.03</v>
+        <v>0.39</v>
       </c>
       <c r="J78" t="s">
         <v>153</v>
@@ -13273,7 +13397,7 @@
         <v>1.2</v>
       </c>
       <c r="L78" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -13284,19 +13408,19 @@
         <v>18</v>
       </c>
       <c r="C79">
-        <v>0.6616</v>
+        <v>0.6617</v>
       </c>
       <c r="D79">
-        <v>0.9947</v>
+        <v>0.9916</v>
       </c>
       <c r="E79">
         <v>0</v>
       </c>
       <c r="F79">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="G79">
-        <v>1.61</v>
+        <v>2.42</v>
       </c>
       <c r="H79">
         <v>104.2600021362305</v>
@@ -13364,16 +13488,16 @@
         <v>100</v>
       </c>
       <c r="C2">
-        <v>1389</v>
+        <v>1418</v>
       </c>
       <c r="D2">
-        <v>836</v>
+        <v>865</v>
       </c>
       <c r="E2">
-        <v>8.359999999999999</v>
+        <v>8.65</v>
       </c>
       <c r="F2">
-        <v>0.9835</v>
+        <v>0.9824000000000001</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -13396,22 +13520,22 @@
         <v>60</v>
       </c>
       <c r="C3">
-        <v>2731.2</v>
+        <v>2741.4</v>
       </c>
       <c r="D3">
-        <v>2281.2</v>
+        <v>2291.4</v>
       </c>
       <c r="E3">
-        <v>38.02</v>
+        <v>38.19</v>
       </c>
       <c r="F3">
-        <v>0.9199000000000001</v>
+        <v>0.9144</v>
       </c>
       <c r="G3">
-        <v>0.7655</v>
+        <v>0.7655999999999999</v>
       </c>
       <c r="H3">
-        <v>0.5305</v>
+        <v>0.5298</v>
       </c>
       <c r="I3">
         <v>1</v>
@@ -13425,19 +13549,19 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <v>3.37</v>
+        <v>3.22</v>
       </c>
       <c r="C4">
-        <v>879.8</v>
+        <v>840.6</v>
       </c>
       <c r="D4">
-        <v>454.14</v>
+        <v>433.6</v>
       </c>
       <c r="E4">
-        <v>134.86</v>
+        <v>134.66</v>
       </c>
       <c r="F4">
-        <v>0.4572</v>
+        <v>0.4547</v>
       </c>
       <c r="G4">
         <v>0</v>

</xml_diff>